<commit_message>
Web pass 4 batch 1: commcare-connect opportunity spine (urls+models)
Web source analysis kicked off (Cal confirmed web scope). 12 functional gaps
from the opportunity URL inventory (~90 endpoints) + model layer: audio
attachments+transcription on visits, granular verification-flag types,
catchment-area verification, form-JSON validation rules, auto-approve-payments,
automatic-visit-verification, archived opportunities, finalize/setup-complete
gate, SMS invite delivery status, org-level payments, sync deliver units, labs.
Web Gap Analysis now 18 rows (12 functional + 6 hygiene).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -11715,7 +11715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="148" min="1" max="1"/>
@@ -12043,6 +12043,534 @@
       <c r="J7" s="171" t="inlineStr">
         <is>
           <t>Pass 1: MTP vs test suite</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-01</t>
+        </is>
+      </c>
+      <c r="B8" s="171" t="inlineStr">
+        <is>
+          <t>Visit verification page</t>
+        </is>
+      </c>
+      <c r="C8" s="171" t="inlineStr">
+        <is>
+          <t>Audio attachments on visits with server-side transcription + translation (AudioAttachment.transcript/translation; audio_attachment/&lt;pk&gt;/transcribe endpoint)</t>
+        </is>
+      </c>
+      <c r="D8" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E8" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (WVV covers image carousel only, not audio/transcription). Src: opportunity AudioAttachment + AudioAttachmentTranscribe</t>
+        </is>
+      </c>
+      <c r="F8" s="171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G8" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H8" s="171" t="inlineStr"/>
+      <c r="I8" s="171" t="inlineStr"/>
+      <c r="J8" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-02</t>
+        </is>
+      </c>
+      <c r="B9" s="171" t="inlineStr">
+        <is>
+          <t>Visit verification page</t>
+        </is>
+      </c>
+      <c r="C9" s="171" t="inlineStr">
+        <is>
+          <t>Granular verification-flag types configured per opportunity: gps, duplicate, location-radius, form-submission time window (start/end), catchment_areas, duration</t>
+        </is>
+      </c>
+      <c r="D9" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E9" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs OD_7 (generic 'verification flags'). Each flag type not a case. Src: OpportunityVerificationFlags model</t>
+        </is>
+      </c>
+      <c r="F9" s="171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G9" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H9" s="171" t="inlineStr"/>
+      <c r="I9" s="171" t="inlineStr"/>
+      <c r="J9" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-03</t>
+        </is>
+      </c>
+      <c r="B10" s="171" t="inlineStr">
+        <is>
+          <t>Visit verification page</t>
+        </is>
+      </c>
+      <c r="C10" s="171" t="inlineStr">
+        <is>
+          <t>Catchment-area based verification: import/export catchment areas (CSV) and flag visits outside the area (CatchmentArea model, import/export_catchment_area)</t>
+        </is>
+      </c>
+      <c r="D10" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E10" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: opportunity CatchmentArea + import_catchment_area/export_catchment_area</t>
+        </is>
+      </c>
+      <c r="F10" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G10" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H10" s="171" t="inlineStr"/>
+      <c r="I10" s="171" t="inlineStr"/>
+      <c r="J10" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-04</t>
+        </is>
+      </c>
+      <c r="B11" s="171" t="inlineStr">
+        <is>
+          <t>Visit verification page</t>
+        </is>
+      </c>
+      <c r="C11" s="171" t="inlineStr">
+        <is>
+          <t>Form-JSON validation rules (question path == value) and per-deliver-unit flag rules (check_attachments, duration) as configurable verification checks</t>
+        </is>
+      </c>
+      <c r="D11" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E11" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: FormJsonValidationRules + DeliverUnitFlagRules + delete_form_json_rule</t>
+        </is>
+      </c>
+      <c r="F11" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G11" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H11" s="171" t="inlineStr"/>
+      <c r="I11" s="171" t="inlineStr"/>
+      <c r="J11" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-05</t>
+        </is>
+      </c>
+      <c r="B12" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C12" s="171" t="inlineStr">
+        <is>
+          <t>auto_approve_payments opportunity setting (distinct from auto_approve_visits) - payments auto-approved without manual step</t>
+        </is>
+      </c>
+      <c r="D12" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E12" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (visit auto-approve covered, payment auto-approve not). Src: Opportunity.auto_approve_payments</t>
+        </is>
+      </c>
+      <c r="F12" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G12" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H12" s="171" t="inlineStr"/>
+      <c r="I12" s="171" t="inlineStr"/>
+      <c r="J12" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-06</t>
+        </is>
+      </c>
+      <c r="B13" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C13" s="171" t="inlineStr">
+        <is>
+          <t>automatic_visit_verification opportunity flag (system auto-verifies visits against rules, distinct from NM manual approve)</t>
+        </is>
+      </c>
+      <c r="D13" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E13" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs MTP. Src: Opportunity.automatic_visit_verification</t>
+        </is>
+      </c>
+      <c r="F13" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G13" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H13" s="171" t="inlineStr"/>
+      <c r="I13" s="171" t="inlineStr"/>
+      <c r="J13" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-07</t>
+        </is>
+      </c>
+      <c r="B14" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity List page</t>
+        </is>
+      </c>
+      <c r="C14" s="171" t="inlineStr">
+        <is>
+          <t>Archived opportunities: an opportunity can be archived (distinct from active/ended); archived-state handling in lists/filters</t>
+        </is>
+      </c>
+      <c r="D14" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E14" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (OLP filters cover Test/Live/Active/Ended, not Archived). Src: Opportunity.archived / is_active</t>
+        </is>
+      </c>
+      <c r="F14" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G14" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H14" s="171" t="inlineStr"/>
+      <c r="I14" s="171" t="inlineStr"/>
+      <c r="J14" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-08</t>
+        </is>
+      </c>
+      <c r="B15" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C15" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity finalize step: an opportunity must be 'setup complete' (payment units + budget + dates) and finalized before going live (OpportunityFinalize / is_setup_complete)</t>
+        </is>
+      </c>
+      <c r="D15" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E15" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (creation covered, finalize/setup-complete gate not). Src: OpportunityFinalize view / Opportunity.is_setup_complete</t>
+        </is>
+      </c>
+      <c r="F15" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G15" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H15" s="171" t="inlineStr"/>
+      <c r="I15" s="171" t="inlineStr"/>
+      <c r="J15" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-09</t>
+        </is>
+      </c>
+      <c r="B16" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C16" s="171" t="inlineStr">
+        <is>
+          <t>Invite SMS delivery status tracking: UserInvite status includes sms_delivered / sms_not_delivered (Twilio delivery callback), plus not_found / invited / accepted</t>
+        </is>
+      </c>
+      <c r="D16" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E16" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs Connect_worker (pending/accepted/not-found). SMS delivered-vs-not not covered. Src: UserInviteStatus</t>
+        </is>
+      </c>
+      <c r="F16" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G16" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H16" s="171" t="inlineStr"/>
+      <c r="I16" s="171" t="inlineStr"/>
+      <c r="J16" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-10</t>
+        </is>
+      </c>
+      <c r="B17" s="171" t="inlineStr">
+        <is>
+          <t>Invoices List page</t>
+        </is>
+      </c>
+      <c r="C17" s="171" t="inlineStr">
+        <is>
+          <t>Organization-level payments to Network Manager orgs (Payment.organization) - distinct from worker payments; incl. payment_method/payment_operator</t>
+        </is>
+      </c>
+      <c r="D17" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E17" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (payment processing covers worker payments only). Src: Payment.organization / payment_method</t>
+        </is>
+      </c>
+      <c r="F17" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G17" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H17" s="171" t="inlineStr"/>
+      <c r="I17" s="171" t="inlineStr"/>
+      <c r="J17" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-11</t>
+        </is>
+      </c>
+      <c r="B18" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity dashboard</t>
+        </is>
+      </c>
+      <c r="C18" s="171" t="inlineStr">
+        <is>
+          <t>Sync deliver units from the HQ app (sync_deliver_units) - refresh deliver-unit definitions from CommCare</t>
+        </is>
+      </c>
+      <c r="D18" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E18" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: sync_deliver_units view</t>
+        </is>
+      </c>
+      <c r="F18" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G18" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H18" s="171" t="inlineStr"/>
+      <c r="I18" s="171" t="inlineStr"/>
+      <c r="J18" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-12</t>
+        </is>
+      </c>
+      <c r="B19" s="171" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C19" s="171" t="inlineStr">
+        <is>
+          <t>Labs/experiments framework (LabsRecord) attached to user/org/opportunity/program - may gate experimental behaviour; confirm if user-facing or internal</t>
+        </is>
+      </c>
+      <c r="D19" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E19" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (possibly internal - reviewer/product to confirm scope). Src: LabsRecord model</t>
+        </is>
+      </c>
+      <c r="F19" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G19" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H19" s="171" t="inlineStr"/>
+      <c r="I19" s="171" t="inlineStr"/>
+      <c r="J19" s="171" t="inlineStr">
+        <is>
+          <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Web batch 2: opportunity views + forms validation rules
10 functional gaps from opportunity views/forms: learn!=deliver app, fields
locked after workers join, managed-opp finalize validations (program budget/date
bounds), add-budget PM-gate + program-cap rules, invoice number uniqueness/
auto-gen, exchange-rate-required, payment-unit date validation, duplicate task-
unit-id, multi-stage opportunity lifecycle. Web Gap Analysis now 28 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -11715,7 +11715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="148" min="1" max="1"/>
@@ -12571,6 +12571,446 @@
       <c r="J19" s="171" t="inlineStr">
         <is>
           <t>Web pass 4/5 batch 1: commcare-connect opportunity spine (urls+models)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-13</t>
+        </is>
+      </c>
+      <c r="B20" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C20" s="171" t="inlineStr">
+        <is>
+          <t>Validation: Learn app and Deliver app cannot be the same app (error on both fields)</t>
+        </is>
+      </c>
+      <c r="D20" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E20" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: OpportunityInitForm.clean</t>
+        </is>
+      </c>
+      <c r="F20" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G20" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H20" s="171" t="inlineStr"/>
+      <c r="I20" s="171" t="inlineStr"/>
+      <c r="J20" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-14</t>
+        </is>
+      </c>
+      <c r="B21" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C21" s="171" t="inlineStr">
+        <is>
+          <t>Certain opportunity fields become non-editable once Connect Workers have joined ('cannot be edited after Connect Workers have joined')</t>
+        </is>
+      </c>
+      <c r="D21" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E21" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: OpportunityInitUpdateForm.clean (_disabled_fields)</t>
+        </is>
+      </c>
+      <c r="F21" s="171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G21" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H21" s="171" t="inlineStr"/>
+      <c r="I21" s="171" t="inlineStr"/>
+      <c r="J21" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-15</t>
+        </is>
+      </c>
+      <c r="B22" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C22" s="171" t="inlineStr">
+        <is>
+          <t>Managed-opp finalize validations: end-date not in past, start-date today-or-later, start&lt;end, both within the program's date window, and total budget (summed across the program's opps) must not exceed program budget</t>
+        </is>
+      </c>
+      <c r="D22" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E22" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs Opp_create_21 (budget page). Program-budget cap + program-date bounds + date rules not cases. Src: OpportunityFinalizeForm.clean</t>
+        </is>
+      </c>
+      <c r="F22" s="171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G22" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H22" s="171" t="inlineStr"/>
+      <c r="I22" s="171" t="inlineStr"/>
+      <c r="J22" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-16</t>
+        </is>
+      </c>
+      <c r="B23" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity dashboard</t>
+        </is>
+      </c>
+      <c r="C23" s="171" t="inlineStr">
+        <is>
+          <t>Add-budget (new workers) rules: PM-only for managed opps; 'users' and 'total budget' can't both be set conflictingly; total budget can't be below already-claimed budget; can't exceed program budget</t>
+        </is>
+      </c>
+      <c r="D23" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E23" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs OD_17. PM-gate + program-cap + not-below-claimed not covered. Src: AddBudgetNewUsersForm.clean</t>
+        </is>
+      </c>
+      <c r="F23" s="171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G23" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H23" s="171" t="inlineStr"/>
+      <c r="I23" s="171" t="inlineStr"/>
+      <c r="J23" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-17</t>
+        </is>
+      </c>
+      <c r="B24" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity dashboard</t>
+        </is>
+      </c>
+      <c r="C24" s="171" t="inlineStr">
+        <is>
+          <t>Add-budget (existing workers) rules: increase can't exceed opportunity remaining budget; must specify visits OR end date; adjustment type required with visits; end date not in past</t>
+        </is>
+      </c>
+      <c r="D24" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E24" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs OD_10-14 (OD_14 decrease-below-completed covered). Budget-exceed + required-field rules not covered. Src: AddBudgetExistingUsersForm.clean</t>
+        </is>
+      </c>
+      <c r="F24" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G24" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H24" s="171" t="inlineStr"/>
+      <c r="I24" s="171" t="inlineStr"/>
+      <c r="J24" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-18</t>
+        </is>
+      </c>
+      <c r="B25" s="171" t="inlineStr">
+        <is>
+          <t>Invoices List page</t>
+        </is>
+      </c>
+      <c r="C25" s="171" t="inlineStr">
+        <is>
+          <t>Invoice number must be unique (reused number rejected) and is auto-generated when left blank</t>
+        </is>
+      </c>
+      <c r="D25" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E25" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: AutomatedPaymentInvoiceForm.clean_invoice_number</t>
+        </is>
+      </c>
+      <c r="F25" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G25" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H25" s="171" t="inlineStr"/>
+      <c r="I25" s="171" t="inlineStr"/>
+      <c r="J25" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-19</t>
+        </is>
+      </c>
+      <c r="B26" s="171" t="inlineStr">
+        <is>
+          <t>Invoices List page</t>
+        </is>
+      </c>
+      <c r="C26" s="171" t="inlineStr">
+        <is>
+          <t>Custom invoice requires an available exchange rate for the chosen date (error if none) and converts via USD toggle (amount &lt;-&gt; amount_usd)</t>
+        </is>
+      </c>
+      <c r="D26" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E26" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs Invoice_04/06. 'Exchange rate not available' error + toggle conversion not covered. Src: AutomatedPaymentInvoiceForm.clean</t>
+        </is>
+      </c>
+      <c r="F26" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G26" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H26" s="171" t="inlineStr"/>
+      <c r="I26" s="171" t="inlineStr"/>
+      <c r="J26" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-20</t>
+        </is>
+      </c>
+      <c r="B27" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C27" s="171" t="inlineStr">
+        <is>
+          <t>Payment unit start/end date validation: end date cannot be earlier than start date</t>
+        </is>
+      </c>
+      <c r="D27" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E27" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: PaymentUnitForm.clean</t>
+        </is>
+      </c>
+      <c r="F27" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G27" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H27" s="171" t="inlineStr"/>
+      <c r="I27" s="171" t="inlineStr"/>
+      <c r="J27" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-21</t>
+        </is>
+      </c>
+      <c r="B28" s="171" t="inlineStr">
+        <is>
+          <t>Re-Learn Task</t>
+        </is>
+      </c>
+      <c r="C28" s="171" t="inlineStr">
+        <is>
+          <t>Adding a task type with a duplicate task-unit ID (already exists for the deliver app) is rejected</t>
+        </is>
+      </c>
+      <c r="D28" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E28" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: AddTaskTypeForm.clean</t>
+        </is>
+      </c>
+      <c r="F28" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G28" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H28" s="171" t="inlineStr"/>
+      <c r="I28" s="171" t="inlineStr"/>
+      <c r="J28" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-22</t>
+        </is>
+      </c>
+      <c r="B29" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity creation</t>
+        </is>
+      </c>
+      <c r="C29" s="171" t="inlineStr">
+        <is>
+          <t>Multi-stage opportunity lifecycle: Init -&gt; InitUpdate -&gt; Finalize, each PM-gated for managed opportunities (role checks + stage transitions)</t>
+        </is>
+      </c>
+      <c r="D29" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E29" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs MTP (creation treated as one flow). Stage/role gating not covered. Src: OpportunityInit/InitUpdate/OpportunityFinalize views</t>
+        </is>
+      </c>
+      <c r="F29" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G29" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H29" s="171" t="inlineStr"/>
+      <c r="I29" s="171" t="inlineStr"/>
+      <c r="J29" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 2: commcare-connect opportunity views + forms</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Web batch 3: opportunity filters + bulk imports
4 gaps: deliver-tab duplicates/review-pending filters + conditional hiding under
auto-verification, bulk visit-status import validations, bulk payment import
(currency/exchange-rate/per-row errors), bulk completed-work import. helpers.py
(dashboard/worker query logic) + tables.py (column defs) skimmed - map to
existing MTP metric/column cases, low new-gap yield. Web Gap Analysis now 32 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -11715,7 +11715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="148" min="1" max="1"/>
@@ -13011,6 +13011,182 @@
       <c r="J29" s="171" t="inlineStr">
         <is>
           <t>Web batch 2: commcare-connect opportunity views + forms</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-23</t>
+        </is>
+      </c>
+      <c r="B30" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C30" s="171" t="inlineStr">
+        <is>
+          <t>Deliver-tab has Has-Duplicates and Deliveries-with-Pending-Review filters, AND both are hidden when the opportunity has automatic_visit_verification enabled (conditional filter set)</t>
+        </is>
+      </c>
+      <c r="D30" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E30" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs Delivery_tab_10-16 (last-active/flags/overlimit). Duplicates + review-pending + conditional hiding missing. Src: DeliverFilterSet</t>
+        </is>
+      </c>
+      <c r="F30" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G30" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H30" s="171" t="inlineStr"/>
+      <c r="I30" s="171" t="inlineStr"/>
+      <c r="J30" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 3: opportunity filters + visit_import + helpers</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-24</t>
+        </is>
+      </c>
+      <c r="B31" s="171" t="inlineStr">
+        <is>
+          <t>Visit verification page</t>
+        </is>
+      </c>
+      <c r="C31" s="171" t="inlineStr">
+        <is>
+          <t>Bulk visit-status import (PM review CSV): per-row status must be a valid VisitValidationStatus, rejection requires a reason, justification required for certain agree/disagree changes, and invalid rows are reported individually</t>
+        </is>
+      </c>
+      <c r="D31" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E31" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs WVV_25-27. Per-row validation + justification-required not covered. Src: bulk_update_visit_status / get_data_by_visit_id</t>
+        </is>
+      </c>
+      <c r="F31" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G31" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H31" s="171" t="inlineStr"/>
+      <c r="I31" s="171" t="inlineStr"/>
+      <c r="J31" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 3: opportunity filters + visit_import + helpers</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-25</t>
+        </is>
+      </c>
+      <c r="B32" s="171" t="inlineStr">
+        <is>
+          <t>Invoices List page</t>
+        </is>
+      </c>
+      <c r="C32" s="171" t="inlineStr">
+        <is>
+          <t>Bulk payment import (CSV): currency must match the opportunity currency, an exchange rate is required/looked up, and invalid rows are reported per-row</t>
+        </is>
+      </c>
+      <c r="D32" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E32" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (payment_import). Src: bulk_update_payments</t>
+        </is>
+      </c>
+      <c r="F32" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G32" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H32" s="171" t="inlineStr"/>
+      <c r="I32" s="171" t="inlineStr"/>
+      <c r="J32" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 3: opportunity filters + visit_import + helpers</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-26</t>
+        </is>
+      </c>
+      <c r="B33" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C33" s="171" t="inlineStr">
+        <is>
+          <t>Bulk completed-work status import (CSV): status validation, rejection reason handling, per-row error reporting, triggers payment-accrued recalculation</t>
+        </is>
+      </c>
+      <c r="D33" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E33" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: bulk_update_completed_work_status</t>
+        </is>
+      </c>
+      <c r="F33" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G33" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H33" s="171" t="inlineStr"/>
+      <c r="I33" s="171" t="inlineStr"/>
+      <c r="J33" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 3: opportunity filters + visit_import + helpers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Web batch 4: program + organization
4 gaps + 1 hygiene: program application reject/decline states, org membership
roles (admin/member) + PM-org permission gating, program invite emails, PM-vs-NM
home dashboards; plus a dead-code finding (is_viewer() references a Role.VIEWER
that does not exist in choices). Web Gap Analysis now 37 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -11715,7 +11715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="148" min="1" max="1"/>
@@ -13187,6 +13187,226 @@
       <c r="J33" s="171" t="inlineStr">
         <is>
           <t>Web batch 3: opportunity filters + visit_import + helpers</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-27</t>
+        </is>
+      </c>
+      <c r="B34" s="171" t="inlineStr">
+        <is>
+          <t>Programs List page</t>
+        </is>
+      </c>
+      <c r="C34" s="171" t="inlineStr">
+        <is>
+          <t>Program application lifecycle includes REJECTED (PM rejects an application) and DECLINED (NM declines an invite) states, in addition to invited/applied/accepted</t>
+        </is>
+      </c>
+      <c r="D34" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E34" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs PLP_02/06/07/16 (invite/apply/accept). Reject + decline paths not covered. Src: program manage_application / apply_or_decline_application</t>
+        </is>
+      </c>
+      <c r="F34" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G34" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H34" s="171" t="inlineStr"/>
+      <c r="I34" s="171" t="inlineStr"/>
+      <c r="J34" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 4: program + organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-28</t>
+        </is>
+      </c>
+      <c r="B35" s="171" t="inlineStr">
+        <is>
+          <t>Programs List page</t>
+        </is>
+      </c>
+      <c r="C35" s="171" t="inlineStr">
+        <is>
+          <t>Organization membership roles (Admin vs Member) and the program-manager-org flag gate access across the web app (e.g. only PM-admins can create programs/invite)</t>
+        </is>
+      </c>
+      <c r="D35" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E35" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (no org-role/permission cases). Src: UserOrganizationMembership.Role / is_program_manager</t>
+        </is>
+      </c>
+      <c r="F35" s="171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G35" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H35" s="171" t="inlineStr"/>
+      <c r="I35" s="171" t="inlineStr"/>
+      <c r="J35" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 4: program + organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-29</t>
+        </is>
+      </c>
+      <c r="B36" s="171" t="inlineStr">
+        <is>
+          <t>Programs List page</t>
+        </is>
+      </c>
+      <c r="C36" s="171" t="inlineStr">
+        <is>
+          <t>Program invite emails: an email is sent when an org is invited to a program, and a notification email to the PM when an org applies</t>
+        </is>
+      </c>
+      <c r="D36" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E36" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: send_program_invite_email / send_program_invite_applied_email</t>
+        </is>
+      </c>
+      <c r="F36" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G36" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H36" s="171" t="inlineStr"/>
+      <c r="I36" s="171" t="inlineStr"/>
+      <c r="J36" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 4: program + organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-30</t>
+        </is>
+      </c>
+      <c r="B37" s="171" t="inlineStr">
+        <is>
+          <t>Programs List page</t>
+        </is>
+      </c>
+      <c r="C37" s="171" t="inlineStr">
+        <is>
+          <t>Role-specific home dashboards: Program Manager vs Network Manager orgs see different landing content/metrics (program_manager_home vs network_manager_home)</t>
+        </is>
+      </c>
+      <c r="D37" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E37" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs PLP_03. Per-role dashboard differences not covered. Src: program_home / program_manager_home / network_manager_home</t>
+        </is>
+      </c>
+      <c r="F37" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G37" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H37" s="171" t="inlineStr"/>
+      <c r="I37" s="171" t="inlineStr"/>
+      <c r="J37" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 4: program + organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="171" t="inlineStr">
+        <is>
+          <t>GAP-MISC-07</t>
+        </is>
+      </c>
+      <c r="B38" s="171" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C38" s="171" t="inlineStr">
+        <is>
+          <t>Possible dead/broken code: UserOrganizationMembership.is_viewer() checks self.Role.VIEWER, but Role only defines ADMIN and MEMBER - calling is_viewer() would raise AttributeError. Confirm whether a VIEWER role is intended or the method is dead.</t>
+        </is>
+      </c>
+      <c r="D38" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E38" s="171" t="inlineStr">
+        <is>
+          <t>Code hygiene finding in web pass. Src: organization/models.py UserOrganizationMembership</t>
+        </is>
+      </c>
+      <c r="F38" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G38" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H38" s="171" t="inlineStr"/>
+      <c r="I38" s="171" t="inlineStr"/>
+      <c r="J38" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 4: program + organization</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Web batch 5: microplanning
3 gaps: work-area file import + async status, automatic work-area status
transitions from visits, async clustering/import polling. Microplanning tab
otherwise well-covered by the MTP (MP_01-40). Web Gap Analysis now 40 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -11715,7 +11715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="148" min="1" max="1"/>
@@ -13407,6 +13407,138 @@
       <c r="J38" s="171" t="inlineStr">
         <is>
           <t>Web batch 4: program + organization</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-31</t>
+        </is>
+      </c>
+      <c r="B39" s="171" t="inlineStr">
+        <is>
+          <t>Microplanning</t>
+        </is>
+      </c>
+      <c r="C39" s="171" t="inlineStr">
+        <is>
+          <t>Work-area file import: upload work areas (WorkAreaImport) with async import-status polling - the ingestion step that precedes clustering/assignment</t>
+        </is>
+      </c>
+      <c r="D39" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E39" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (MP cases assume areas already uploaded). Src: microplanning WorkAreaImport / import_status</t>
+        </is>
+      </c>
+      <c r="F39" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G39" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H39" s="171" t="inlineStr"/>
+      <c r="I39" s="171" t="inlineStr"/>
+      <c r="J39" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 5: microplanning</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-32</t>
+        </is>
+      </c>
+      <c r="B40" s="171" t="inlineStr">
+        <is>
+          <t>Microplanning</t>
+        </is>
+      </c>
+      <c r="C40" s="171" t="inlineStr">
+        <is>
+          <t>Automatic work-area status transitions driven by visits: NOT_VISITED -&gt; VISITED on first approved visit, -&gt; EXPECTED_VISIT_REACHED when approved visit count hits the expected count</t>
+        </is>
+      </c>
+      <c r="D40" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E40" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs MP_07/08 (statuses listed, transitions not). Src: WorkArea.update_status</t>
+        </is>
+      </c>
+      <c r="F40" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G40" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H40" s="171" t="inlineStr"/>
+      <c r="I40" s="171" t="inlineStr"/>
+      <c r="J40" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 5: microplanning</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-33</t>
+        </is>
+      </c>
+      <c r="B41" s="171" t="inlineStr">
+        <is>
+          <t>Microplanning</t>
+        </is>
+      </c>
+      <c r="C41" s="171" t="inlineStr">
+        <is>
+          <t>Clustering and import run as async jobs with status polling (cluster_work_areas + clustering_status; import + import_status) - UI must poll for completion</t>
+        </is>
+      </c>
+      <c r="D41" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E41" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs MP_02. Async/polling behaviour not covered. Src: cluster_work_areas / clustering_status</t>
+        </is>
+      </c>
+      <c r="F41" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G41" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H41" s="171" t="inlineStr"/>
+      <c r="I41" s="171" t="inlineStr"/>
+      <c r="J41" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 5: microplanning</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Web batch 6: users + commcarehq + audit + reports + flags; web source pass complete
6 gaps: SMS status callback, web accept-invite/redirect flow, web feature-flag
admin, full audit-reports workflow (feature-gated), reporting/KPI module, credential
issuance model. Login covered by MTP Login tab; commcarehq covered by Opp_create
API cases. WEB SOURCE PASS COMPLETE. Web Gap Analysis now 46 rows.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -11715,7 +11715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="148" min="1" max="1"/>
@@ -13539,6 +13539,270 @@
       <c r="J41" s="171" t="inlineStr">
         <is>
           <t>Web batch 5: microplanning</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-34</t>
+        </is>
+      </c>
+      <c r="B42" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C42" s="171" t="inlineStr">
+        <is>
+          <t>SMS status callback (Twilio) endpoint updates invite delivery status to sms_delivered / sms_not_delivered on the UserInvite</t>
+        </is>
+      </c>
+      <c r="D42" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E42" s="171" t="inlineStr">
+        <is>
+          <t>Backs SRC-W-09; callback endpoint itself untested. Src: users SMSStatusCallbackView</t>
+        </is>
+      </c>
+      <c r="F42" s="171" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G42" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H42" s="171" t="inlineStr"/>
+      <c r="I42" s="171" t="inlineStr"/>
+      <c r="J42" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 6: users + commcarehq + audit + reports + flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-35</t>
+        </is>
+      </c>
+      <c r="B43" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity List page</t>
+        </is>
+      </c>
+      <c r="C43" s="171" t="inlineStr">
+        <is>
+          <t>Web accept-invite / invite-redirect link flow (opening an opportunity invite URL lands on accept view / redirects into the opportunity)</t>
+        </is>
+      </c>
+      <c r="D43" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E43" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (invite acceptance treated as mobile-only). Src: AcceptInviteView / InviteRedirectView</t>
+        </is>
+      </c>
+      <c r="F43" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G43" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H43" s="171" t="inlineStr"/>
+      <c r="I43" s="171" t="inlineStr"/>
+      <c r="J43" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 6: users + commcarehq + audit + reports + flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-36</t>
+        </is>
+      </c>
+      <c r="B44" s="171" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C44" s="171" t="inlineStr">
+        <is>
+          <t>Web feature-flag administration: enable/disable feature flags and waffle switches from the web (feature_flags / toggle_switch / update_flag)</t>
+        </is>
+      </c>
+      <c r="D44" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E44" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP. Src: flags/views.py</t>
+        </is>
+      </c>
+      <c r="F44" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G44" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H44" s="171" t="inlineStr"/>
+      <c r="I44" s="171" t="inlineStr"/>
+      <c r="J44" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 6: users + commcarehq + audit + reports + flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-37</t>
+        </is>
+      </c>
+      <c r="B45" s="171" t="inlineStr">
+        <is>
+          <t>Opportunity dashboard</t>
+        </is>
+      </c>
+      <c r="C45" s="171" t="inlineStr">
+        <is>
+          <t>Audit reports workflow (feature-flag-gated): list audit reports, view detail, act on per-entry tasks, complete a report, export - beyond the single Audit-opportunity button</t>
+        </is>
+      </c>
+      <c r="D45" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E45" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs OD_2 (audit button only). Full audit workflow untested. Src: audit/views.py</t>
+        </is>
+      </c>
+      <c r="F45" s="171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G45" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H45" s="171" t="inlineStr"/>
+      <c r="I45" s="171" t="inlineStr"/>
+      <c r="J45" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 6: users + commcarehq + audit + reports + flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-38</t>
+        </is>
+      </c>
+      <c r="B46" s="171" t="inlineStr">
+        <is>
+          <t>Cross-cutting</t>
+        </is>
+      </c>
+      <c r="C46" s="171" t="inlineStr">
+        <is>
+          <t>Reporting module: Delivery Stats / KPI reports and Invoice reports with filters + CSV/XLSX export (org-level analytics)</t>
+        </is>
+      </c>
+      <c r="D46" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E46" s="171" t="inlineStr">
+        <is>
+          <t>MISSING from MTP (no reports/KPI cases). Src: reports/views.py DeliveryStatsReportView / InvoiceReportView</t>
+        </is>
+      </c>
+      <c r="F46" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G46" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H46" s="171" t="inlineStr"/>
+      <c r="I46" s="171" t="inlineStr"/>
+      <c r="J46" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 6: users + commcarehq + audit + reports + flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="171" t="inlineStr">
+        <is>
+          <t>GAP-SRC-W-39</t>
+        </is>
+      </c>
+      <c r="B47" s="171" t="inlineStr">
+        <is>
+          <t>App Credentials</t>
+        </is>
+      </c>
+      <c r="C47" s="171" t="inlineStr">
+        <is>
+          <t>UserCredential issuance with Learn/Delivery credential levels + types + issued_on + computed titles (drives credential-gated opportunity access)</t>
+        </is>
+      </c>
+      <c r="D47" s="171" t="inlineStr">
+        <is>
+          <t>🟡 Automatable - not yet done</t>
+        </is>
+      </c>
+      <c r="E47" s="171" t="inlineStr">
+        <is>
+          <t>PARTIAL vs Credentials_1-3 + Worker History. Level/type issuance model not covered. Src: users/models UserCredential</t>
+        </is>
+      </c>
+      <c r="F47" s="171" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G47" s="171" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+      <c r="H47" s="171" t="inlineStr"/>
+      <c r="I47" s="171" t="inlineStr"/>
+      <c r="J47" s="171" t="inlineStr">
+        <is>
+          <t>Web batch 6: users + commcarehq + audit + reports + flags</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update web MTP: mark Opportunity List + Programs List automation status
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -31609,9 +31609,17 @@
 - Created program is shown on the programs list page</t>
         </is>
       </c>
-      <c r="E2" s="66" t="n"/>
+      <c r="E2" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F2" s="67" t="n"/>
-      <c r="G2" s="67" t="n"/>
+      <c r="G2" s="67" t="inlineStr">
+        <is>
+          <t>Automated (setup flow: create_program)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="67" t="inlineStr">
@@ -31635,9 +31643,17 @@
           <t xml:space="preserve">User should be able to invite the NMs to the programs </t>
         </is>
       </c>
-      <c r="E3" s="66" t="n"/>
+      <c r="E3" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F3" s="67" t="n"/>
-      <c r="G3" s="67" t="n"/>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>Automated (setup flow: invite_network_manager)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="67" t="inlineStr">
@@ -31668,9 +31684,17 @@
 </t>
         </is>
       </c>
-      <c r="E4" s="66" t="n"/>
+      <c r="E4" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F4" s="67" t="n"/>
-      <c r="G4" s="67" t="n"/>
+      <c r="G4" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (card summary fields)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="67" t="inlineStr">
@@ -31694,9 +31718,17 @@
 </t>
         </is>
       </c>
-      <c r="E5" s="66" t="n"/>
+      <c r="E5" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F5" s="67" t="n"/>
-      <c r="G5" s="67" t="n"/>
+      <c r="G5" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (View Status expand)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="67" t="inlineStr">
@@ -31724,9 +31756,17 @@
 - Number Accepted</t>
         </is>
       </c>
-      <c r="E6" s="66" t="n"/>
+      <c r="E6" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F6" s="67" t="n"/>
-      <c r="G6" s="67" t="n"/>
+      <c r="G6" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (acceptance_funnel)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="67" t="inlineStr">
@@ -31754,9 +31794,17 @@
 </t>
         </is>
       </c>
-      <c r="E7" s="66" t="n"/>
+      <c r="E7" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F7" s="67" t="n"/>
-      <c r="G7" s="67" t="n"/>
+      <c r="G7" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (nm_application_statuses)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="67" t="inlineStr">
@@ -31785,9 +31833,17 @@
 - View Opportunity </t>
         </is>
       </c>
-      <c r="E8" s="66" t="n"/>
+      <c r="E8" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F8" s="67" t="n"/>
-      <c r="G8" s="67" t="n"/>
+      <c r="G8" s="67" t="inlineStr">
+        <is>
+          <t>Automated (setup flow: Create/View Opportunity when accepted)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="67" t="inlineStr">
@@ -31810,7 +31866,11 @@
       </c>
       <c r="E9" s="66" t="n"/>
       <c r="F9" s="67" t="n"/>
-      <c r="G9" s="67" t="n"/>
+      <c r="G9" s="67" t="inlineStr">
+        <is>
+          <t>Not on list page; = Recent Activities destinations (link targets asserted)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="67" t="inlineStr">
@@ -31836,7 +31896,11 @@
       </c>
       <c r="E10" s="66" t="n"/>
       <c r="F10" s="67" t="n"/>
-      <c r="G10" s="67" t="n"/>
+      <c r="G10" s="67" t="inlineStr">
+        <is>
+          <t>Covered via Opportunity List PM columns (test_olp_list_page)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="67" t="inlineStr">
@@ -31862,9 +31926,17 @@
 - The accepted status appears after Opportunity creation, so confirm that as well</t>
         </is>
       </c>
-      <c r="E11" s="66" t="n"/>
+      <c r="E11" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F11" s="67" t="n"/>
-      <c r="G11" s="67" t="n"/>
+      <c r="G11" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (card summary fields)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="67" t="inlineStr">
@@ -31890,9 +31962,17 @@
           <t xml:space="preserve">- If there are any opportunities in a program, user should be able to see the list of all opportunities by clicking the button </t>
         </is>
       </c>
-      <c r="E12" s="66" t="n"/>
+      <c r="E12" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F12" s="67" t="n"/>
-      <c r="G12" s="67" t="n"/>
+      <c r="G12" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (click_view_opportunities)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="67" t="inlineStr">
@@ -31915,9 +31995,17 @@
 - The number of items in the list should be restricted to 3 per category</t>
         </is>
       </c>
-      <c r="E13" s="66" t="n"/>
+      <c r="E13" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F13" s="67" t="n"/>
-      <c r="G13" s="67" t="n"/>
+      <c r="G13" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (Recent Activities categories + rows)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="67" t="inlineStr">
@@ -31943,9 +32031,17 @@
 - When user clicks on an Opportunity under ‘Pending Payments’, they should jump to the Worker List page with the payment tab open</t>
         </is>
       </c>
-      <c r="E14" s="66" t="n"/>
+      <c r="E14" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F14" s="67" t="n"/>
-      <c r="G14" s="67" t="n"/>
+      <c r="G14" s="67" t="inlineStr">
+        <is>
+          <t>Automated (link target asserted): Recent Activities row hrefs</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="67" t="inlineStr">
@@ -31971,9 +32067,17 @@
 - When user clicks on an Opportunity under ‘Inactive Workers’, they should jump to the Worker List page with the filtered list of workers who have not delivered any visits or not completed a learning module in the last 3 days.</t>
         </is>
       </c>
-      <c r="E15" s="66" t="n"/>
+      <c r="E15" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F15" s="67" t="n"/>
-      <c r="G15" s="67" t="n"/>
+      <c r="G15" s="67" t="inlineStr">
+        <is>
+          <t>Automated (link target asserted): Recent Activities row hrefs</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="67" t="inlineStr">
@@ -32000,9 +32104,17 @@
           <t xml:space="preserve">- Program manager should be able to see if someone applies for a program </t>
         </is>
       </c>
-      <c r="E16" s="66" t="n"/>
+      <c r="E16" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F16" s="67" t="n"/>
-      <c r="G16" s="67" t="n"/>
+      <c r="G16" s="67" t="inlineStr">
+        <is>
+          <t>Automated (setup flow: apply_to_program)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="67" t="inlineStr">
@@ -32028,9 +32140,17 @@
           <t>- User is able to see the opportunities related to specific NM user</t>
         </is>
       </c>
-      <c r="E17" s="66" t="n"/>
+      <c r="E17" s="66" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F17" s="67" t="n"/>
-      <c r="G17" s="67" t="n"/>
+      <c r="G17" s="67" t="inlineStr">
+        <is>
+          <t>Automated: test_plp_list_page (View Opportunities)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E17">
@@ -33024,9 +33144,17 @@
 - Opportunities should be listed in the order of start date </t>
         </is>
       </c>
-      <c r="E2" s="69" t="n"/>
+      <c r="E2" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F2" s="73" t="n"/>
-      <c r="G2" s="73" t="n"/>
+      <c r="G2" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (verify_loaded)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="73" t="inlineStr">
@@ -33047,7 +33175,11 @@
       </c>
       <c r="E3" s="69" t="n"/>
       <c r="F3" s="73" t="n"/>
-      <c r="G3" s="73" t="n"/>
+      <c r="G3" s="73" t="inlineStr">
+        <is>
+          <t>Not automated - stale (no Add New button on current list page)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="73" t="inlineStr">
@@ -33074,9 +33206,17 @@
 - User should also see "Add New" button </t>
         </is>
       </c>
-      <c r="E4" s="69" t="n"/>
+      <c r="E4" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F4" s="73" t="n"/>
-      <c r="G4" s="73" t="n"/>
+      <c r="G4" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (landing)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="73" t="inlineStr">
@@ -33118,9 +33258,17 @@
 - User should be able to sort the list by clicking on any column header </t>
         </is>
       </c>
-      <c r="E5" s="69" t="n"/>
+      <c r="E5" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F5" s="73" t="n"/>
-      <c r="G5" s="73" t="n"/>
+      <c r="G5" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (PM+NM columns, sortable headers)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="73" t="n"/>
@@ -33199,7 +33347,11 @@
       </c>
       <c r="E7" s="69" t="n"/>
       <c r="F7" s="73" t="n"/>
-      <c r="G7" s="73" t="n"/>
+      <c r="G7" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: filter behaviour)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="73" t="inlineStr">
@@ -33226,9 +33378,17 @@
 - User should be able to navigate forward backwards using the pagination arrows  </t>
         </is>
       </c>
-      <c r="E8" s="69" t="n"/>
+      <c r="E8" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F8" s="73" t="n"/>
-      <c r="G8" s="73" t="n"/>
+      <c r="G8" s="73" t="inlineStr">
+        <is>
+          <t>Automated: rows-per-page control (multi-page nav = Tier 2)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="73" t="inlineStr">
@@ -33249,9 +33409,17 @@
         </is>
       </c>
       <c r="D9" s="68" t="n"/>
-      <c r="E9" s="69" t="n"/>
+      <c r="E9" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F9" s="73" t="n"/>
-      <c r="G9" s="73" t="n"/>
+      <c r="G9" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (open_opportunity)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="73" t="inlineStr">
@@ -33280,9 +33448,17 @@
 </t>
         </is>
       </c>
-      <c r="E10" s="69" t="n"/>
+      <c r="E10" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F10" s="73" t="n"/>
-      <c r="G10" s="73" t="n"/>
+      <c r="G10" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (filter modal fields)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="73" t="inlineStr">
@@ -33311,9 +33487,17 @@
 - Non test opportunities should be displayed when 'no' is selected</t>
         </is>
       </c>
-      <c r="E11" s="69" t="n"/>
+      <c r="E11" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F11" s="73" t="n"/>
-      <c r="G11" s="73" t="n"/>
+      <c r="G11" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (is_test options)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="73" t="inlineStr">
@@ -33344,9 +33528,17 @@
 - Inactive opportunities should be displayed when inactive is selected</t>
         </is>
       </c>
-      <c r="E12" s="69" t="n"/>
+      <c r="E12" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F12" s="73" t="n"/>
-      <c r="G12" s="73" t="n"/>
+      <c r="G12" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (status options)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="73" t="inlineStr">
@@ -33373,9 +33565,17 @@
 - Opportunities that are part of selected program should be displayed</t>
         </is>
       </c>
-      <c r="E13" s="69" t="n"/>
+      <c r="E13" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F13" s="73" t="n"/>
-      <c r="G13" s="73" t="n"/>
+      <c r="G13" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (program options, PM)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="73" t="inlineStr">
@@ -33404,7 +33604,11 @@
       </c>
       <c r="E14" s="69" t="n"/>
       <c r="F14" s="73" t="n"/>
-      <c r="G14" s="73" t="n"/>
+      <c r="G14" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: apply + filter badge)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="73" t="inlineStr">
@@ -33434,7 +33638,11 @@
       </c>
       <c r="E15" s="69" t="n"/>
       <c r="F15" s="73" t="n"/>
-      <c r="G15" s="73" t="n"/>
+      <c r="G15" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: multi-select status)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="73" t="inlineStr">
@@ -33464,7 +33672,11 @@
       </c>
       <c r="E16" s="69" t="n"/>
       <c r="F16" s="73" t="n"/>
-      <c r="G16" s="73" t="n"/>
+      <c r="G16" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: multi-select program)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="73" t="inlineStr">
@@ -33492,7 +33704,11 @@
       </c>
       <c r="E17" s="69" t="n"/>
       <c r="F17" s="73" t="n"/>
-      <c r="G17" s="73" t="n"/>
+      <c r="G17" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: filter persistence)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="73" t="inlineStr">
@@ -33523,9 +33739,17 @@
 View Invoices </t>
         </is>
       </c>
-      <c r="E18" s="69" t="n"/>
+      <c r="E18" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F18" s="73" t="n"/>
-      <c r="G18" s="73" t="n"/>
+      <c r="G18" s="73" t="inlineStr">
+        <is>
+          <t>Automated: test_olp_list_page (kebab_options)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="73" t="inlineStr">
@@ -33551,7 +33775,11 @@
       </c>
       <c r="E19" s="69" t="n"/>
       <c r="F19" s="73" t="n"/>
-      <c r="G19" s="73" t="n"/>
+      <c r="G19" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: kebab nav target)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="73" t="inlineStr">
@@ -33577,7 +33805,11 @@
       </c>
       <c r="E20" s="69" t="n"/>
       <c r="F20" s="73" t="n"/>
-      <c r="G20" s="73" t="n"/>
+      <c r="G20" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: kebab nav target)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="73" t="inlineStr">
@@ -33603,7 +33835,11 @@
       </c>
       <c r="E21" s="69" t="n"/>
       <c r="F21" s="73" t="n"/>
-      <c r="G21" s="73" t="n"/>
+      <c r="G21" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: kebab nav target)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="73" t="inlineStr">
@@ -33631,7 +33867,11 @@
       </c>
       <c r="E22" s="69" t="n"/>
       <c r="F22" s="73" t="n"/>
-      <c r="G22" s="73" t="n"/>
+      <c r="G22" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 2: combined filters)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="73" t="inlineStr">
@@ -33659,7 +33899,11 @@
       </c>
       <c r="E23" s="69" t="n"/>
       <c r="F23" s="73" t="n"/>
-      <c r="G23" s="73" t="n"/>
+      <c r="G23" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 3: pending-invites drill-down)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="73" t="inlineStr">
@@ -33686,7 +33930,11 @@
       </c>
       <c r="E24" s="69" t="n"/>
       <c r="F24" s="73" t="n"/>
-      <c r="G24" s="73" t="n"/>
+      <c r="G24" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 3: inactive-workers drill-down)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="73" t="inlineStr">
@@ -33713,7 +33961,11 @@
       </c>
       <c r="E25" s="69" t="n"/>
       <c r="F25" s="73" t="n"/>
-      <c r="G25" s="73" t="n"/>
+      <c r="G25" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 3: payments-due drill-down)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="73" t="inlineStr">
@@ -33740,7 +33992,11 @@
       </c>
       <c r="E26" s="69" t="n"/>
       <c r="F26" s="73" t="n"/>
-      <c r="G26" s="73" t="n"/>
+      <c r="G26" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 3: active-workers drill-down)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="73" t="inlineStr">
@@ -33767,7 +34023,11 @@
       </c>
       <c r="E27" s="69" t="n"/>
       <c r="F27" s="73" t="n"/>
-      <c r="G27" s="73" t="n"/>
+      <c r="G27" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 3: total-deliveries drill-down)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="73" t="inlineStr">
@@ -33794,7 +34054,11 @@
       </c>
       <c r="E28" s="69" t="n"/>
       <c r="F28" s="73" t="n"/>
-      <c r="G28" s="73" t="n"/>
+      <c r="G28" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 3: verified-deliveries drill-down)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="73" t="inlineStr">
@@ -33821,7 +34085,11 @@
       </c>
       <c r="E29" s="69" t="n"/>
       <c r="F29" s="73" t="n"/>
-      <c r="G29" s="73" t="n"/>
+      <c r="G29" s="73" t="inlineStr">
+        <is>
+          <t>Pending (Tier 3: worker-earnings drill-down)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E29">

</xml_diff>

<commit_message>
Opportunity List: Tier 2 filter behaviour + Tier 3 drill-downs
Follow-up to the list-page Tier 1 work. Live-green on staging.

- test_olp_list_behaviour: PM journey - status filter (single + multi),
  program filter, combined is_test+status, filter persistence across
  navigate-away/back, pagination (guarded), and PM count-cell drill-downs
  keyed by the sort param the table renderer appends
  (OLP_06/07/13/14/15/16/22/27/28/29/30)
- test_olp_list_page (NM): assert NM count-cell drill-downs
  (OLP_23/24/26) and kebab action targets by href (OLP_17/18/19/20)
- page object + locators: status badges, stats/count links, combined
  filter, kebab hrefs
- web MTP: mark the above OLP cases automated

Only OLP_02 remains uncovered (stale - no Add New button on the list page).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -33345,11 +33345,15 @@
 Ended </t>
         </is>
       </c>
-      <c r="E7" s="69" t="n"/>
+      <c r="E7" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F7" s="73" t="n"/>
       <c r="G7" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: filter behaviour)</t>
+          <t>Automated: test_olp_list_behaviour (status filter)</t>
         </is>
       </c>
     </row>
@@ -33386,7 +33390,7 @@
       <c r="F8" s="73" t="n"/>
       <c r="G8" s="73" t="inlineStr">
         <is>
-          <t>Automated: rows-per-page control (multi-page nav = Tier 2)</t>
+          <t>Automated: test_olp_list_behaviour (pagination; skips when &lt;=20 opps)</t>
         </is>
       </c>
     </row>
@@ -33602,11 +33606,15 @@
 - Number of filters selected should be displayed on the filters icon</t>
         </is>
       </c>
-      <c r="E14" s="69" t="n"/>
+      <c r="E14" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F14" s="73" t="n"/>
       <c r="G14" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: apply + filter badge)</t>
+          <t>Automated: test_olp_list_behaviour (apply + filter badge)</t>
         </is>
       </c>
     </row>
@@ -33636,11 +33644,15 @@
           <t>- Multiple filters selected should be applied on the opportunities</t>
         </is>
       </c>
-      <c r="E15" s="69" t="n"/>
+      <c r="E15" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F15" s="73" t="n"/>
       <c r="G15" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: multi-select status)</t>
+          <t>Automated: test_olp_list_behaviour (multi-select status)</t>
         </is>
       </c>
     </row>
@@ -33670,11 +33682,15 @@
           <t>- Opportunities related to the selected programs should be displayed</t>
         </is>
       </c>
-      <c r="E16" s="69" t="n"/>
+      <c r="E16" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F16" s="73" t="n"/>
       <c r="G16" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: multi-select program)</t>
+          <t>Automated: test_olp_list_behaviour (program filter)</t>
         </is>
       </c>
     </row>
@@ -33702,11 +33718,15 @@
           <t>- Applied filters should be preserved when user navigate away and back</t>
         </is>
       </c>
-      <c r="E17" s="69" t="n"/>
+      <c r="E17" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F17" s="73" t="n"/>
       <c r="G17" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: filter persistence)</t>
+          <t>Automated: test_olp_list_behaviour (filter persistence)</t>
         </is>
       </c>
     </row>
@@ -33773,11 +33793,15 @@
           <t>- User should be land on opportunity dashboard</t>
         </is>
       </c>
-      <c r="E19" s="69" t="n"/>
+      <c r="E19" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F19" s="73" t="n"/>
       <c r="G19" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: kebab nav target)</t>
+          <t>Automated: test_olp_list_behaviour (kebab View Opportunity target)</t>
         </is>
       </c>
     </row>
@@ -33803,11 +33827,15 @@
           <t>- User should be land on Connect workers page</t>
         </is>
       </c>
-      <c r="E20" s="69" t="n"/>
+      <c r="E20" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F20" s="73" t="n"/>
       <c r="G20" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: kebab nav target)</t>
+          <t>Automated: test_olp_list_behaviour (kebab View Connect Workers target)</t>
         </is>
       </c>
     </row>
@@ -33833,11 +33861,15 @@
           <t>- User should be land on invoices page</t>
         </is>
       </c>
-      <c r="E21" s="69" t="n"/>
+      <c r="E21" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F21" s="73" t="n"/>
       <c r="G21" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: kebab nav target)</t>
+          <t>Automated: test_olp_list_behaviour (kebab View Invoices target)</t>
         </is>
       </c>
     </row>
@@ -33865,11 +33897,15 @@
           <t>- Opportunities based on the selected filters should be displayed</t>
         </is>
       </c>
-      <c r="E22" s="69" t="n"/>
+      <c r="E22" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F22" s="73" t="n"/>
       <c r="G22" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 2: combined filters)</t>
+          <t>Automated: test_olp_list_behaviour (combined is_test + status)</t>
         </is>
       </c>
     </row>
@@ -33897,11 +33933,15 @@
           <t>- User should be able to land on connect workers page and view the pending invites first</t>
         </is>
       </c>
-      <c r="E23" s="69" t="n"/>
+      <c r="E23" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F23" s="73" t="n"/>
       <c r="G23" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 3: pending-invites drill-down)</t>
+          <t>Automated: test_olp_list_page NM (Pending Invites count cell present)</t>
         </is>
       </c>
     </row>
@@ -33928,11 +33968,15 @@
           <t>- User should be able to land on connect workers page and view the Inactive workers</t>
         </is>
       </c>
-      <c r="E24" s="69" t="n"/>
+      <c r="E24" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F24" s="73" t="n"/>
       <c r="G24" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 3: inactive-workers drill-down)</t>
+          <t>Automated: test_olp_list_page NM (Inactive workers drill-down)</t>
         </is>
       </c>
     </row>
@@ -33959,11 +34003,15 @@
           <t>- User should be able to land on the payments tab and view the pending payments</t>
         </is>
       </c>
-      <c r="E25" s="69" t="n"/>
+      <c r="E25" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F25" s="73" t="n"/>
       <c r="G25" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 3: payments-due drill-down)</t>
+          <t>Automated: test_olp_list_page NM (Payments Due drill-down)</t>
         </is>
       </c>
     </row>
@@ -33990,11 +34038,15 @@
           <t>- User should be able to land on connect workers page</t>
         </is>
       </c>
-      <c r="E26" s="69" t="n"/>
+      <c r="E26" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F26" s="73" t="n"/>
       <c r="G26" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 3: active-workers drill-down)</t>
+          <t>Automated: test_olp_list_behaviour (Active workers count cell)</t>
         </is>
       </c>
     </row>
@@ -34021,11 +34073,15 @@
           <t>- User should be able to land on delivery tab and view the pending approvals</t>
         </is>
       </c>
-      <c r="E27" s="69" t="n"/>
+      <c r="E27" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F27" s="73" t="n"/>
       <c r="G27" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 3: total-deliveries drill-down)</t>
+          <t>Automated: test_olp_list_behaviour (Total Deliveries drill-down)</t>
         </is>
       </c>
     </row>
@@ -34052,11 +34108,15 @@
           <t xml:space="preserve">- User should be able to land on delivery tab </t>
         </is>
       </c>
-      <c r="E28" s="69" t="n"/>
+      <c r="E28" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F28" s="73" t="n"/>
       <c r="G28" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 3: verified-deliveries drill-down)</t>
+          <t>Automated: test_olp_list_behaviour (Verified Deliveries drill-down)</t>
         </is>
       </c>
     </row>
@@ -34083,11 +34143,15 @@
           <t xml:space="preserve">- User should be able to land on the payments tab </t>
         </is>
       </c>
-      <c r="E29" s="69" t="n"/>
+      <c r="E29" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F29" s="73" t="n"/>
       <c r="G29" s="73" t="inlineStr">
         <is>
-          <t>Pending (Tier 3: worker-earnings drill-down)</t>
+          <t>Automated: test_olp_list_behaviour (Worker Earnings drill-down)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
OLP: leave OLP_02 manual; note NM drill-downs skip without NM data
OLP_02 (NM cannot create): the only create path is the program-scoped
ManagedOpportunityInit, which resolves the program in setup() before the
ProgramManagerMixin check - a clean 403 needs a real program slug the NM
org lacks on staging (bogus slug 500s). Left manual with rationale.

Also flag in the MTP that the NM count drill-downs (OLP_23/24/26) skip
when the NM org has no opportunities (currently the case on staging), so
they are coded but not yet live-verified.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -33177,7 +33177,7 @@
       <c r="F3" s="73" t="n"/>
       <c r="G3" s="73" t="inlineStr">
         <is>
-          <t>Not automated - stale (no Add New button on current list page)</t>
+          <t>Manual - only create path is program-scoped ManagedOpportunityInit; clean 403 needs a real program slug the NM org lacks on staging (bogus slug 500s)</t>
         </is>
       </c>
     </row>
@@ -33941,7 +33941,7 @@
       <c r="F23" s="73" t="n"/>
       <c r="G23" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (Pending Invites count cell present)</t>
+          <t>Automated: test_olp_list_page NM (skips when NM org has no opportunities - unverified on staging)</t>
         </is>
       </c>
     </row>
@@ -33976,7 +33976,7 @@
       <c r="F24" s="73" t="n"/>
       <c r="G24" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (Inactive workers drill-down)</t>
+          <t>Automated: test_olp_list_page NM (skips when NM org has no opportunities - unverified on staging)</t>
         </is>
       </c>
     </row>
@@ -34011,7 +34011,7 @@
       <c r="F25" s="73" t="n"/>
       <c r="G25" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (Payments Due drill-down)</t>
+          <t>Automated: test_olp_list_page NM (skips when NM org has no opportunities - unverified on staging)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
OLP_02: automate NM create-denial (403) via managed opportunity-init
The managed opportunity-init view resolves the program by program_id (UUID)
then denies non-PM orgs with 403 (ProgramManagerMixin). Probe it as the NM
org using a seeded staging program_id (OLP Test program); skips where no
program_id is configured for the env (prod). Update web MTP.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -33173,11 +33173,15 @@
           <t>-User is not able to create an opportunity as NM user</t>
         </is>
       </c>
-      <c r="E3" s="69" t="n"/>
+      <c r="E3" s="69" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="F3" s="73" t="n"/>
       <c r="G3" s="73" t="inlineStr">
         <is>
-          <t>Manual - only create path is program-scoped ManagedOpportunityInit; clean 403 needs a real program slug the NM org lacks on staging (bogus slug 500s)</t>
+          <t>Automated: test_olp_list_page NM (managed opportunity-init returns 403 for NM; uses seeded program_id)</t>
         </is>
       </c>
     </row>
@@ -33941,7 +33945,7 @@
       <c r="F23" s="73" t="n"/>
       <c r="G23" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (skips when NM org has no opportunities - unverified on staging)</t>
+          <t>Automated: test_olp_list_page NM (Pending Invites count cell) - runs only when NM list has rows</t>
         </is>
       </c>
     </row>
@@ -33976,7 +33980,7 @@
       <c r="F24" s="73" t="n"/>
       <c r="G24" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (skips when NM org has no opportunities - unverified on staging)</t>
+          <t>Automated: test_olp_list_page NM (Inactive workers drill-down) - runs only when NM list has rows</t>
         </is>
       </c>
     </row>
@@ -34011,7 +34015,7 @@
       <c r="F25" s="73" t="n"/>
       <c r="G25" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (skips when NM org has no opportunities - unverified on staging)</t>
+          <t>Automated: test_olp_list_page NM (Payments Due drill-down) - runs only when NM list has rows</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
OLP: fix row locator (even/odd not group) + robust filter/kebab/pagination
Critical: opportunity-list rows render class even/odd (django-tables2), not the
template's literal 'group' - so the old row locator matched nothing and every
row-dependent assertion (filters, drill-downs, kebab, pagination) was silently
skip-guarded, making the Tier 2/3 tests pass vacuously. Now verified live.

- row locators keyed on even/odd; match opportunity name by contains (the name
  cell also carries the NM org as a subtitle line)
- filter selection sets the native <select> + syncs TomSelect via its instance
  (reliable for multi-select, unlike clicking dropdown options)
- pagination navigates via ?page=N (the pager's own goToPage path)
- kebab reads scoped to the target row (every row's dropdown is in the DOM)
- next/prev page buttons matched by chevron icon
- MTP: OLP_23/24/26 now verified with seeded OLP_Test_Opp

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -33945,7 +33945,7 @@
       <c r="F23" s="73" t="n"/>
       <c r="G23" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (Pending Invites count cell) - runs only when NM list has rows</t>
+          <t>Automated: test_olp_list_page NM (Pending Invites count cell) - verified with seeded OLP_Test_Opp</t>
         </is>
       </c>
     </row>
@@ -33980,7 +33980,7 @@
       <c r="F24" s="73" t="n"/>
       <c r="G24" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (Inactive workers drill-down) - runs only when NM list has rows</t>
+          <t>Automated: test_olp_list_page NM (Inactive workers drill-down) - verified with seeded OLP_Test_Opp</t>
         </is>
       </c>
     </row>
@@ -34015,7 +34015,7 @@
       <c r="F25" s="73" t="n"/>
       <c r="G25" s="73" t="inlineStr">
         <is>
-          <t>Automated: test_olp_list_page NM (Payments Due drill-down) - runs only when NM list has rows</t>
+          <t>Automated: test_olp_list_page NM (Payments Due drill-down) - verified with seeded OLP_Test_Opp</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MTP: annotate Opportunity Dashboard cases with automation status
Add Comments to the "Opportunity dashboard" tab recording where each Tier 2/3
case stands:
- OD_9/10/11/12/13/14/16/17: automated (PR #38) with the test refs.
- OD_8 and OD_15: WEB half automated; MOBILE half (push/notification history;
  device visit reflection) is out of web scope - needs a Maestro mobile hybrid
  test (enrolled worker + BrowserStack + new flow, @on_demand).
- OD_36: automated (catchment export/import).
- OD_44 and OD_46: partially automated - the PM "Review Sheet" export option and
  the visit-status import are hidden when automatic_visit_verification is ON.
  Both current staging opps (Demo Opportunity, Add Budget Opp) are auto-verify
  (verified 2026-09-02), so those paths are BLOCKED pending a manual-verification
  staging opp.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -1959,7 +1959,11 @@
       </c>
       <c r="E9" s="66" t="n"/>
       <c r="F9" s="123" t="n"/>
-      <c r="G9" s="123" t="n"/>
+      <c r="G9" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Web part automated (Send Message page reachable) - PR #38, tests/test_opd_budget.py::test_opd_08_send_message_page. MOBILE HALF NOT AUTOMATED (push notification on device + notification history) - out of web/Playwright scope; needs a Maestro mobile hybrid test (device signs in as the enrolled worker after the web send, like TASKING_HYBRID / test_e2e_relearn_lifecycle). Prereqs: enrolled mobile worker on the opp, BrowserStack/Appium, a new Maestro flow; runs @on_demand.</t>
+        </is>
+      </c>
       <c r="H9" s="123" t="n"/>
       <c r="I9" s="123" t="n"/>
     </row>
@@ -1991,7 +1995,11 @@
       </c>
       <c r="E10" s="66" t="n"/>
       <c r="F10" s="123" t="n"/>
-      <c r="G10" s="123" t="n"/>
+      <c r="G10" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget.py::test_opd_09_add_connect_workers_redirect (redirects to user_invite; #id_users present).</t>
+        </is>
+      </c>
       <c r="H10" s="123" t="n"/>
       <c r="I10" s="123" t="n"/>
     </row>
@@ -2023,7 +2031,11 @@
       </c>
       <c r="E11" s="66" t="n"/>
       <c r="F11" s="123" t="n"/>
-      <c r="G11" s="123" t="n"/>
+      <c r="G11" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget_mutations.py::test_opd_10 (increase visits; Max Visits reflects; mutate-then-revert on the dedicated staging Add Budget opp; net-zero).</t>
+        </is>
+      </c>
       <c r="H11" s="123" t="n"/>
       <c r="I11" s="123" t="n"/>
     </row>
@@ -2055,7 +2067,11 @@
       </c>
       <c r="E12" s="66" t="n"/>
       <c r="F12" s="123" t="n"/>
-      <c r="G12" s="123" t="n"/>
+      <c r="G12" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget_mutations.py::test_opd_11_increase_visits_proportional (delta = N x payment units; net-zero).</t>
+        </is>
+      </c>
       <c r="H12" s="123" t="n"/>
       <c r="I12" s="123" t="n"/>
     </row>
@@ -2087,7 +2103,11 @@
       </c>
       <c r="E13" s="66" t="n"/>
       <c r="F13" s="123" t="n"/>
-      <c r="G13" s="123" t="n"/>
+      <c r="G13" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget_mutations.py::test_opd_12_decrease_visits_proportional (net-zero increase-then-decrease).</t>
+        </is>
+      </c>
       <c r="H13" s="123" t="n"/>
       <c r="I13" s="123" t="n"/>
     </row>
@@ -2119,7 +2139,11 @@
       </c>
       <c r="E14" s="66" t="n"/>
       <c r="F14" s="123" t="n"/>
-      <c r="G14" s="123" t="n"/>
+      <c r="G14" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget.py::test_opd_13_negative_visits_validation (number_of_visits min=1 via browser ValidityState).</t>
+        </is>
+      </c>
       <c r="H14" s="123" t="n"/>
       <c r="I14" s="123" t="n"/>
     </row>
@@ -2149,7 +2173,11 @@
       </c>
       <c r="E15" s="66" t="n"/>
       <c r="F15" s="123" t="n"/>
-      <c r="G15" s="123" t="n"/>
+      <c r="G15" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget_mutations.py::test_opd_14 (decrease below completed/zero rejected with 'Cannot decrease...' error; no change). Exercised via a below-zero decrease (same validation/message); the exact below-COMPLETED path additionally needs a worker with completed visits.</t>
+        </is>
+      </c>
       <c r="H15" s="123" t="n"/>
       <c r="I15" s="123" t="n"/>
     </row>
@@ -2178,7 +2206,11 @@
       </c>
       <c r="E16" s="66" t="n"/>
       <c r="F16" s="123" t="n"/>
-      <c r="G16" s="123" t="n"/>
+      <c r="G16" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Web reflection automated (Connect Workers/Deliver max-visit denominators) - PR #38, test_opd_budget_mutations.py::test_opd_15_change_reflected_on_connect_workers. MOBILE REFLECTION NOT AUTOMATED (updated visit count on the device) - out of web scope; needs the same Maestro mobile hybrid follow-up as OD_8.</t>
+        </is>
+      </c>
       <c r="H16" s="123" t="n"/>
       <c r="I16" s="123" t="n"/>
     </row>
@@ -2208,7 +2240,11 @@
       </c>
       <c r="E17" s="66" t="n"/>
       <c r="F17" s="123" t="n"/>
-      <c r="G17" s="123" t="n"/>
+      <c r="G17" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget.py::test_opd_16_confirm_modal_shows_computed_visits (totalVisits shown in the confirm modal; no submit).</t>
+        </is>
+      </c>
       <c r="H17" s="123" t="n"/>
       <c r="I17" s="123" t="n"/>
     </row>
@@ -2240,7 +2276,11 @@
       </c>
       <c r="E18" s="66" t="n"/>
       <c r="F18" s="123" t="n"/>
-      <c r="G18" s="123" t="n"/>
+      <c r="G18" s="123" t="inlineStr">
+        <is>
+          <t>AUTOMATION: Automated - PR #38, test_opd_budget.py::test_opd_17_new_workers_autocalc_total_budget (total_budget auto-updates with the new-worker count).</t>
+        </is>
+      </c>
       <c r="H18" s="123" t="n"/>
       <c r="I18" s="123" t="n"/>
     </row>
@@ -2863,7 +2903,7 @@
       <c r="F38" s="188" t="inlineStr"/>
       <c r="G38" s="189" t="inlineStr">
         <is>
-          <t>Added from source-derived gap analysis (2026-08-26), beyond documented OD_1-OD_19. Src: opportunity_menu.html:27-39; dashboard.html:111-114.</t>
+          <t>Added from source-derived gap analysis (2026-08-26), beyond documented OD_1-OD_19. Src: opportunity_menu.html:27-39; dashboard.html:111-114. | AUTOMATION: Automated - PR #38, tests/test_opd_exports.py (catchment Export queues a background task; Import with missing columns rejected). Non-mutating.</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3142,7 @@
       <c r="F46" s="188" t="inlineStr"/>
       <c r="G46" s="189" t="inlineStr">
         <is>
-          <t>Added from source-derived gap analysis (2026-08-26), beyond documented OD_1-OD_19. Src: views.py:2753-2774, 536-602; deliver.html:36-84.</t>
+          <t>Added from source-derived gap analysis (2026-08-26), beyond documented OD_1-OD_19. Src: views.py:2753-2774, 536-602; deliver.html:36-84. | AUTOMATION: Partially automated - PR #38, test_opd_exports.py::test_opd_44_deliver_export_flow. NM 'User Visits Sheet' option + export form verified; the background export queue is best-effort (required-heavy HTMX form). PM 'PM Review Sheet' is hidden when automatic_visit_verification is ON - both current staging opps (Demo Opportunity, Add Budget Opp) are auto-verify, verified 2026-09-02 - so the PM path can't run live yet. BLOCKED: needs a manual-verification (auto-verify OFF) staging opp.</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3206,7 @@
       <c r="F48" s="188" t="inlineStr"/>
       <c r="G48" s="189" t="inlineStr">
         <is>
-          <t>Added from source-derived gap analysis (2026-08-26), beyond documented OD_1-OD_19. Src: views.py:614-615; payments.html:18.</t>
+          <t>Added from source-derived gap analysis (2026-08-26), beyond documented OD_1-OD_19. Src: views.py:614-615; payments.html:18. | AUTOMATION: Partially automated - PR #38, tests/test_opd_exports.py. Payments import rejects non-csv/xlsx ('File format not supported') - automated. Visit-status import is hidden under automatic_visit_verification (skips on current auto-verify staging opps). BLOCKED: needs a manual-verification staging opp.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Note Batch A/B automation progress in MTP ledger
Add the 7 worker-module cases automated this session that were not yet in the
"Automation (existing MTP)" tab: Connect_worker_17 (sort), Delivery_tab_10/11/
13/14/16 (deliver-tab filters) and Payment Processing_2, each marked
automated with its Playwright test reference.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -20025,7 +20025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G317"/>
+  <dimension ref="A1:G324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="148" min="1" max="1"/>
@@ -31763,6 +31763,265 @@
       <c r="G317" s="171" t="inlineStr">
         <is>
           <t>QA-owned (UI/e2e - eng cannot cover)</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_17</t>
+        </is>
+      </c>
+      <c r="B318" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C318" s="171" t="inlineStr">
+        <is>
+          <t>Verify user can sort the workers list by clicking the header columns</t>
+        </is>
+      </c>
+      <c r="D318" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E318" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_list_view.py::test_connect_worker_17_sort_list_by_header</t>
+        </is>
+      </c>
+      <c r="F318" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch A/B (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G318" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="171" t="inlineStr">
+        <is>
+          <t>Delivery_tab_10</t>
+        </is>
+      </c>
+      <c r="B319" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C319" s="171" t="inlineStr">
+        <is>
+          <t>Verify Filters pop up modal is displayed by clicking the filters icon on the delivery tab</t>
+        </is>
+      </c>
+      <c r="D319" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E319" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_deliver_filters.py::test_delivery_tab_10_filter_modal_opens</t>
+        </is>
+      </c>
+      <c r="F319" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch A/B (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G319" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="171" t="inlineStr">
+        <is>
+          <t>Delivery_tab_11</t>
+        </is>
+      </c>
+      <c r="B320" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C320" s="171" t="inlineStr">
+        <is>
+          <t>Verify Last active filter dropdown contains the expected options (Any time / 1 / 3 / 7 days ago)</t>
+        </is>
+      </c>
+      <c r="D320" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E320" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_deliver_filters.py::test_delivery_tab_11_last_active_options</t>
+        </is>
+      </c>
+      <c r="F320" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch A/B (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G320" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="171" t="inlineStr">
+        <is>
+          <t>Delivery_tab_13</t>
+        </is>
+      </c>
+      <c r="B321" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C321" s="171" t="inlineStr">
+        <is>
+          <t>Verify Deliveries-with-flags filter dropdown contains the expected options (---------/Yes/No)</t>
+        </is>
+      </c>
+      <c r="D321" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E321" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_deliver_filters.py::test_delivery_tab_13_deliveries_with_flags_options</t>
+        </is>
+      </c>
+      <c r="F321" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch A/B (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G321" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="171" t="inlineStr">
+        <is>
+          <t>Delivery_tab_14</t>
+        </is>
+      </c>
+      <c r="B322" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C322" s="171" t="inlineStr">
+        <is>
+          <t>Verify Has-overlimit-deliveries filter dropdown contains the expected options (---------/Yes/No)</t>
+        </is>
+      </c>
+      <c r="D322" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E322" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_deliver_filters.py::test_delivery_tab_14_has_overlimit_options</t>
+        </is>
+      </c>
+      <c r="F322" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch A/B (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G322" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="171" t="inlineStr">
+        <is>
+          <t>Delivery_tab_16</t>
+        </is>
+      </c>
+      <c r="B323" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C323" s="171" t="inlineStr">
+        <is>
+          <t>Ensure all filter combinations are applied simultaneously and function correctly (badge counts them)</t>
+        </is>
+      </c>
+      <c r="D323" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E323" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_deliver_filters.py::test_delivery_tab_16_filter_combination_applies</t>
+        </is>
+      </c>
+      <c r="F323" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch A/B (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G323" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="171" t="inlineStr">
+        <is>
+          <t>Payment Processing_2</t>
+        </is>
+      </c>
+      <c r="B324" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C324" s="171" t="inlineStr">
+        <is>
+          <t>Confirm user sees a message when a payment is made (covered via the import-confirmation path; confirm "Pay button" wording w/ product)</t>
+        </is>
+      </c>
+      <c r="D324" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E324" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_payments.py::test_payment_processing_01_02_03_04</t>
+        </is>
+      </c>
+      <c r="F324" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch A/B (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G324" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automate Learn_tab_04 (assessment Passed) + log it in MTP ledger
Batch D probe found covid_opp_test has workers with a Passed assessment, so
Learn_tab_04 is automatable read-only now: verify_passed_assessment_worker
finds a Passed row and asserts 100% modules completed with non-empty Attempts
and Completed Learning (ported from the Selenium verify_worker_assessment_status).
Learn_tab_03 (Failed) still needs a seeded failed-assessment worker.

Validated headed against staging: 1/1 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -20025,7 +20025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G324"/>
+  <dimension ref="A1:G325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="148" min="1" max="1"/>
@@ -32020,6 +32020,43 @@
         </is>
       </c>
       <c r="G324" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="171" t="inlineStr">
+        <is>
+          <t>Learn_tab_04</t>
+        </is>
+      </c>
+      <c r="B325" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C325" s="171" t="inlineStr">
+        <is>
+          <t>Verify Assessment status is shown as Passed when a worker passes the assessment (100% modules, attempts + completed learning present)</t>
+        </is>
+      </c>
+      <c r="D325" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E325" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_list_view.py::test_learn_tab_04_assessment_passed</t>
+        </is>
+      </c>
+      <c r="F325" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch D probe (feature/workers-web-automation, 2026-09-09)</t>
+        </is>
+      </c>
+      <c r="G325" s="171" t="inlineStr">
         <is>
           <t>Already automated (n/a)</t>
         </is>

</xml_diff>

<commit_message>
Automate Connect_worker_02/_03 invite cases (Batch C phase 1)
Zero-mutation invite-lifecycle cases that read an existing pending invite on the
Connect Workers tab (no SMS sent):
- Connect_worker_02: a not-yet-accepted invite shows the 'Invite pending' status.
- Connect_worker_03: Resend/Delete buttons enable only when an invite is selected
  (select then deselect, asserting the disabled<->enabled flip).

Adds invite-lifecycle locators (add-worker, resend/delete toolbar, invite input +
submit, pending indicator, delete-confirm) and logs both cases in the MTP ledger.
Validated headed against staging: 2/2 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -20025,7 +20025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G325"/>
+  <dimension ref="A1:G327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="148" min="1" max="1"/>
@@ -32057,6 +32057,80 @@
         </is>
       </c>
       <c r="G325" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_02</t>
+        </is>
+      </c>
+      <c r="B326" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C326" s="171" t="inlineStr">
+        <is>
+          <t>Verify user is able to see the status as invite pending until the invitation is accepted</t>
+        </is>
+      </c>
+      <c r="D326" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E326" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_invites.py::test_connect_worker_02_pending_invite_status</t>
+        </is>
+      </c>
+      <c r="F326" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C phase 1 (feature/workers-web-automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G326" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_03</t>
+        </is>
+      </c>
+      <c r="B327" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C327" s="171" t="inlineStr">
+        <is>
+          <t>Verify resend/delete invite buttons are enabled only when the user selects the invites</t>
+        </is>
+      </c>
+      <c r="D327" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E327" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_invites.py::test_connect_worker_03_resend_delete_gated_by_selection</t>
+        </is>
+      </c>
+      <c r="F327" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C phase 1 (feature/workers-web-automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G327" s="171" t="inlineStr">
         <is>
           <t>Already automated (n/a)</t>
         </is>

</xml_diff>

<commit_message>
Automate Connect_worker_04/_07 + Learn_tab_03 on seeded data (Batch C)
Anshu seeded Worker_Lifecycle_Automation with accepted (Case_list), suspended
(Map_08), pending, and failed-assessment (Map_09) workers. New read-only tests
against exact live values:
- _04: accepted worker shows 'Invite accepted'
- _07: suspended worker shows 'User suspended'
- Learn_tab_03: Map_09 shows Assessment 'Failed'

Adds verify_worker_status / verify_assessment_status and a WORKER_LIFECYCLE test
data block (statuses/phones read from the app; reserved numbers recorded). Note:
demo numbers do not enforce the 24h cooldown, so _09/_10 stay manual.
Validated headed: 3/3 pass. _04 + Learn_tab_03 logged in the MTP ledger.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -20025,7 +20025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G330"/>
+  <dimension ref="A1:G332"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="148" min="1" max="1"/>
@@ -32242,6 +32242,80 @@
         </is>
       </c>
       <c r="G330" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_04</t>
+        </is>
+      </c>
+      <c r="B331" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C331" s="171" t="inlineStr">
+        <is>
+          <t>Verify worker status is updated to invite accepted when the invitation is accepted</t>
+        </is>
+      </c>
+      <c r="D331" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E331" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_04_accepted_status</t>
+        </is>
+      </c>
+      <c r="F331" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C seeded data (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G331" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="171" t="inlineStr">
+        <is>
+          <t>Learn_tab_03</t>
+        </is>
+      </c>
+      <c r="B332" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C332" s="171" t="inlineStr">
+        <is>
+          <t>Verify Assessment status is shown as Failed when the worker fails the assessment</t>
+        </is>
+      </c>
+      <c r="D332" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E332" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_learn_tab_03_assessment_failed</t>
+        </is>
+      </c>
+      <c r="F332" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C seeded data (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G332" s="171" t="inlineStr">
         <is>
           <t>Already automated (n/a)</t>
         </is>

</xml_diff>

<commit_message>
Automate Connect_worker_10/_11/_14 resend gating (Batch C)
Resend behaviour on the seeded Worker_Lifecycle_Automation opportunity (all
non-destructive - resend of accepted/suspended is skipped, demo numbers are not
actually re-messaged):
- _10: resending a pending invite -> "Successfully resent 1 invite(s)."
- _11: resending an accepted worker -> "skipped, as they have already accepted"
- _14: resending a suspended worker -> skipped

Adds resend_worker_and_message (re-navigates to the workers list, since resend
redirects to the dashboard). Logged in the MTP ledger. Validated headed: 6/6 pass
(with _04/_07/Learn_tab_03).

_09 (24h cooldown) stays manual: demo numbers do not enforce the cooldown.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -20025,7 +20025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G332"/>
+  <dimension ref="A1:G335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="148" min="1" max="1"/>
@@ -32316,6 +32316,117 @@
         </is>
       </c>
       <c r="G332" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_10</t>
+        </is>
+      </c>
+      <c r="B333" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C333" s="171" t="inlineStr">
+        <is>
+          <t>Verify user is able to resend the invite for invite-pending workers (Successfully resent)</t>
+        </is>
+      </c>
+      <c r="D333" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E333" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_10_resend_allowed_for_pending</t>
+        </is>
+      </c>
+      <c r="F333" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C seeded data (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G333" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_11</t>
+        </is>
+      </c>
+      <c r="B334" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C334" s="171" t="inlineStr">
+        <is>
+          <t>Verify user is not able to resend the invite for accepted workers (skipped - already accepted)</t>
+        </is>
+      </c>
+      <c r="D334" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E334" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_11_resend_skipped_for_accepted</t>
+        </is>
+      </c>
+      <c r="F334" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C seeded data (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G334" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_14</t>
+        </is>
+      </c>
+      <c r="B335" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C335" s="171" t="inlineStr">
+        <is>
+          <t>Verify user is not able to resend the invite for suspended users (skipped)</t>
+        </is>
+      </c>
+      <c r="D335" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E335" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_14_resend_skipped_for_suspended</t>
+        </is>
+      </c>
+      <c r="F335" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C seeded data (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G335" s="171" t="inlineStr">
         <is>
           <t>Already automated (n/a)</t>
         </is>

</xml_diff>

<commit_message>
Automate Connect_worker_15 bulk resend messages (Batch C)
Bulk-resend a mix of worker states on Worker_Lifecycle_Automation and assert the
combined result: accepted/suspended are skipped ("already accepted") while the
pending invite is resent ("Successfully resent"). Non-destructive. Adds
select_worker_rows / bulk_resend_and_message. Logged in the MTP ledger.
Validated headed: 1/1 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -20025,7 +20025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G335"/>
+  <dimension ref="A1:G336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="148" min="1" max="1"/>
@@ -32427,6 +32427,43 @@
         </is>
       </c>
       <c r="G335" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_15</t>
+        </is>
+      </c>
+      <c r="B336" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C336" s="171" t="inlineStr">
+        <is>
+          <t>Verify appropriate messages are displayed when the user bulk-resends invites to a mix of worker types (accepted/suspended skipped, pending resent)</t>
+        </is>
+      </c>
+      <c r="D336" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E336" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_15_bulk_resend_messages</t>
+        </is>
+      </c>
+      <c r="F336" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C seeded data (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G336" s="171" t="inlineStr">
         <is>
           <t>Already automated (n/a)</t>
         </is>

</xml_diff>

<commit_message>
Annotate Connect Workers plan tab with automation status
Fill the Comments column for all 37 Connect-workers-tab cases: the automated
ones name their Playwright test; the remaining ones carry the reason they are
not automated (async not-found for _06/_13, manual-only 24h cooldown for _09,
destructive bulk-delete for _16, mobile-required Learn_tab_02, delivery-
completion logic for Delivery_tab_06/07).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -464,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="191">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -971,6 +971,9 @@
     <xf numFmtId="0" fontId="31" fillId="23" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3364,7 +3367,11 @@
       </c>
       <c r="E3" s="66" t="n"/>
       <c r="F3" s="80" t="n"/>
-      <c r="G3" s="80" t="n"/>
+      <c r="G3" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_wlv_01_02_03 (migration)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="73" t="n"/>
@@ -3408,7 +3415,11 @@
       </c>
       <c r="E5" s="66" t="n"/>
       <c r="F5" s="85" t="n"/>
-      <c r="G5" s="85" t="n"/>
+      <c r="G5" s="88" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_invites.py::test_connect_worker_02_pending_invite_status</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="73" t="inlineStr">
@@ -3436,7 +3447,11 @@
       </c>
       <c r="E6" s="66" t="n"/>
       <c r="F6" s="80" t="n"/>
-      <c r="G6" s="80" t="n"/>
+      <c r="G6" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_invites.py::test_connect_worker_03_resend_delete_gated_by_selection</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="73" t="inlineStr">
@@ -3457,7 +3472,11 @@
       </c>
       <c r="E7" s="66" t="n"/>
       <c r="F7" s="104" t="n"/>
-      <c r="G7" s="104" t="n"/>
+      <c r="G7" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_lifecycle.py::test_connect_worker_04_accepted_status (Worker_Lifecycle_Automation)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="73" t="inlineStr">
@@ -3487,7 +3506,11 @@
       </c>
       <c r="E8" s="66" t="n"/>
       <c r="F8" s="104" t="n"/>
-      <c r="G8" s="80" t="n"/>
+      <c r="G8" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_invites.py::test_connect_worker_05_12_08_invite_resend_delete</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="73" t="inlineStr">
@@ -3517,7 +3540,11 @@
       </c>
       <c r="E9" s="66" t="n"/>
       <c r="F9" s="104" t="n"/>
-      <c r="G9" s="80" t="n"/>
+      <c r="G9" s="68" t="inlineStr">
+        <is>
+          <t>⏳ Not automated - not-found "mobile under Name" resolves asynchronously (SMS delivery callback); a freshly-invited number shows "—". Needs a resolved not-found worker seeded (requested from data setup).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="73" t="inlineStr">
@@ -3546,7 +3573,11 @@
       </c>
       <c r="E10" s="66" t="n"/>
       <c r="F10" s="85" t="n"/>
-      <c r="G10" s="85" t="n"/>
+      <c r="G10" s="88" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_lifecycle.py::test_connect_worker_07_suspended_status (+ suspend/revoke action in test_worker_visit_verification.py)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="73" t="inlineStr">
@@ -3576,7 +3607,11 @@
       </c>
       <c r="E11" s="66" t="n"/>
       <c r="F11" s="85" t="n"/>
-      <c r="G11" s="85" t="n"/>
+      <c r="G11" s="88" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_invites.py::test_connect_worker_05_12_08_invite_resend_delete</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="73" t="inlineStr">
@@ -3605,7 +3640,11 @@
       </c>
       <c r="E12" s="66" t="n"/>
       <c r="F12" s="85" t="n"/>
-      <c r="G12" s="85" t="n"/>
+      <c r="G12" s="88" t="inlineStr">
+        <is>
+          <t>🔴 Manual only - demo/reserved numbers do NOT enforce the 24h resend cooldown (per data setup); needs a real number to verify.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="73" t="inlineStr">
@@ -3634,7 +3673,11 @@
       </c>
       <c r="E13" s="66" t="n"/>
       <c r="F13" s="80" t="n"/>
-      <c r="G13" s="85" t="n"/>
+      <c r="G13" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_lifecycle.py::test_connect_worker_10_resend_allowed_for_pending</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="73" t="inlineStr">
@@ -3664,7 +3707,11 @@
       </c>
       <c r="E14" s="66" t="n"/>
       <c r="F14" s="85" t="n"/>
-      <c r="G14" s="85" t="n"/>
+      <c r="G14" s="88" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_lifecycle.py::test_connect_worker_11_resend_skipped_for_accepted</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="73" t="inlineStr">
@@ -3693,7 +3740,11 @@
       </c>
       <c r="E15" s="66" t="n"/>
       <c r="F15" s="85" t="n"/>
-      <c r="G15" s="85" t="n"/>
+      <c r="G15" s="88" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_invites.py::test_connect_worker_05_12_08_invite_resend_delete</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="73" t="inlineStr">
@@ -3722,7 +3773,11 @@
       </c>
       <c r="E16" s="66" t="n"/>
       <c r="F16" s="85" t="n"/>
-      <c r="G16" s="85" t="n"/>
+      <c r="G16" s="88" t="inlineStr">
+        <is>
+          <t>⏳ Not automated - delete not-found shares the async not-found dependency as _06; needs a resolved not-found worker seeded.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="73" t="inlineStr">
@@ -3752,7 +3807,11 @@
       </c>
       <c r="E17" s="66" t="n"/>
       <c r="F17" s="85" t="n"/>
-      <c r="G17" s="85" t="n"/>
+      <c r="G17" s="88" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_lifecycle.py::test_connect_worker_14_resend_skipped_for_suspended</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="73" t="inlineStr">
@@ -3785,7 +3844,11 @@
       </c>
       <c r="E18" s="66" t="n"/>
       <c r="F18" s="104" t="n"/>
-      <c r="G18" s="104" t="n"/>
+      <c r="G18" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_lifecycle.py::test_connect_worker_15_bulk_resend_messages</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="73" t="inlineStr">
@@ -3816,7 +3879,11 @@
       </c>
       <c r="E19" s="66" t="n"/>
       <c r="F19" s="104" t="n"/>
-      <c r="G19" s="104" t="n"/>
+      <c r="G19" s="118" t="inlineStr">
+        <is>
+          <t>⏸ Deferred - bulk delete across all types would delete the seeded pending/accepted workers (destructive). Not automated to protect the seed.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="73" t="inlineStr">
@@ -3849,7 +3916,11 @@
       </c>
       <c r="E20" s="66" t="n"/>
       <c r="F20" s="80" t="n"/>
-      <c r="G20" s="80" t="n"/>
+      <c r="G20" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_connect_worker_17_sort_list_by_header</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="12.75" customHeight="1" s="148">
       <c r="A21" s="76" t="n"/>
@@ -3896,7 +3967,11 @@
       </c>
       <c r="E22" s="66" t="n"/>
       <c r="F22" s="80" t="n"/>
-      <c r="G22" s="80" t="n"/>
+      <c r="G22" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_wlv_01_02_03 (migration)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="73" t="inlineStr">
@@ -3924,7 +3999,11 @@
       </c>
       <c r="E23" s="66" t="n"/>
       <c r="F23" s="80" t="n"/>
-      <c r="G23" s="80" t="n"/>
+      <c r="G23" s="68" t="inlineStr">
+        <is>
+          <t>🔴 Not automated (web) - requires a mobile learn-app submission during the test; web-only cannot drive it.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="73" t="inlineStr">
@@ -3952,7 +4031,11 @@
       </c>
       <c r="E24" s="66" t="n"/>
       <c r="F24" s="80" t="n"/>
-      <c r="G24" s="80" t="n"/>
+      <c r="G24" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_lifecycle.py::test_learn_tab_03_assessment_failed (Map_09)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="73" t="inlineStr">
@@ -3980,7 +4063,11 @@
       </c>
       <c r="E25" s="66" t="n"/>
       <c r="F25" s="80" t="n"/>
-      <c r="G25" s="80" t="n"/>
+      <c r="G25" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_learn_tab_04_assessment_passed</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="12.75" customHeight="1" s="148">
       <c r="A26" s="76" t="n"/>
@@ -4021,7 +4108,11 @@
       </c>
       <c r="E27" s="66" t="n"/>
       <c r="F27" s="80" t="n"/>
-      <c r="G27" s="80" t="n"/>
+      <c r="G27" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_wlv_01_02_03 (Deliver tab, migration)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="73" t="inlineStr">
@@ -4051,7 +4142,11 @@
       </c>
       <c r="E28" s="66" t="n"/>
       <c r="F28" s="80" t="n"/>
-      <c r="G28" s="80" t="n"/>
+      <c r="G28" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_wlv_01_02_03 (deliver headers)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="73" t="inlineStr">
@@ -4083,7 +4178,11 @@
       </c>
       <c r="E29" s="66" t="n"/>
       <c r="F29" s="80" t="n"/>
-      <c r="G29" s="80" t="n"/>
+      <c r="G29" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_wlv_04_worker_status_count_breakdown (Delivered)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="73" t="inlineStr">
@@ -4112,7 +4211,11 @@
       </c>
       <c r="E30" s="66" t="n"/>
       <c r="F30" s="80" t="n"/>
-      <c r="G30" s="80" t="n"/>
+      <c r="G30" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_wlv_04/05 (Approved breakdown)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="73" t="inlineStr">
@@ -4141,7 +4244,11 @@
       </c>
       <c r="E31" s="66" t="n"/>
       <c r="F31" s="80" t="n"/>
-      <c r="G31" s="80" t="n"/>
+      <c r="G31" s="190" t="inlineStr">
+        <is>
+          <t>⏸ Deferred - delivery-completion logic (1 visit per payment unit); eng-covered, needs controlled visit data.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="73" t="inlineStr">
@@ -4170,7 +4277,11 @@
       </c>
       <c r="E32" s="66" t="n"/>
       <c r="F32" s="80" t="n"/>
-      <c r="G32" s="80" t="n"/>
+      <c r="G32" s="68" t="inlineStr">
+        <is>
+          <t>⏸ Deferred - delivery-completion rule (required + optional approved); eng-covered, needs controlled visit data.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="73" t="inlineStr">
@@ -4204,7 +4315,11 @@
       </c>
       <c r="E33" s="66" t="n"/>
       <c r="F33" s="80" t="n"/>
-      <c r="G33" s="80" t="n"/>
+      <c r="G33" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_list_view.py::test_wlv_04/05 (Rejected breakdown)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="73" t="inlineStr">
@@ -4241,7 +4356,11 @@
       </c>
       <c r="E34" s="66" t="n"/>
       <c r="F34" s="104" t="n"/>
-      <c r="G34" s="80" t="n"/>
+      <c r="G34" s="68" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_deliver_filters.py::test_delivery_tab_10_filter_modal_opens</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="73" t="inlineStr">
@@ -4278,7 +4397,11 @@
       </c>
       <c r="E35" s="66" t="n"/>
       <c r="F35" s="104" t="n"/>
-      <c r="G35" s="104" t="n"/>
+      <c r="G35" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_deliver_filters.py::test_delivery_tab_11_last_active_options</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="73" t="inlineStr">
@@ -4311,7 +4434,11 @@
       </c>
       <c r="E36" s="66" t="n"/>
       <c r="F36" s="104" t="n"/>
-      <c r="G36" s="104" t="n"/>
+      <c r="G36" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_deliver_filters.py::test_delivery_tab_13_deliveries_with_flags_options</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="73" t="inlineStr">
@@ -4344,7 +4471,11 @@
       </c>
       <c r="E37" s="66" t="n"/>
       <c r="F37" s="104" t="n"/>
-      <c r="G37" s="104" t="n"/>
+      <c r="G37" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_deliver_filters.py::test_delivery_tab_14_has_overlimit_options</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="73" t="inlineStr">
@@ -4374,7 +4505,11 @@
       </c>
       <c r="E38" s="66" t="n"/>
       <c r="F38" s="104" t="n"/>
-      <c r="G38" s="104" t="n"/>
+      <c r="G38" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_deliver_filters.py::test_delivery_tab_16_filter_combination_applies</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="12.75" customHeight="1" s="148">
       <c r="A39" s="76" t="n"/>
@@ -4419,6 +4554,11 @@
         </is>
       </c>
       <c r="E40" s="66" t="n"/>
+      <c r="G40" s="83" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_payments.py::test_payment_processing_01_02_03_04</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="82" t="inlineStr">
@@ -4438,6 +4578,11 @@
         </is>
       </c>
       <c r="E41" s="66" t="n"/>
+      <c r="G41" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_payments.py (import-confirmation path)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="82" t="inlineStr">
@@ -4469,6 +4614,11 @@
         </is>
       </c>
       <c r="E42" s="66" t="n"/>
+      <c r="G42" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_payments.py (last-paid history popup)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="82" t="inlineStr">
@@ -4498,6 +4648,11 @@
         </is>
       </c>
       <c r="E43" s="66" t="n"/>
+      <c r="G43" s="118" t="inlineStr">
+        <is>
+          <t>✅ Automated (Playwright, feature/workers-web-automation): test_worker_payments.py (rollback)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Automate gap cases GAP-SRC-W-46/49/52 (worker gaps, group 1)
Read-only gap-derived cases against covid_opp_test:
- _46: the per-worker profile page shows its KPI header tiles (Total Visits /
  Pending Tasks / Rejected Visits / Accrued / Paid).
- _49: the Work Area Assignments tab is present and its page is reachable (HTTP
  200) under MICROPLANNING (on for covid_opp_test). Off-state (tab absent + 404)
  needs a non-microplanning opp.
- _52: the Payments currency columns carry a currency-code suffix ('Accrued
  (INR)' etc.). Footer sums / import cache-lock remain eng-covered.

Plan-sheet Comments updated for these three rows. Validated headed: 3/3 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -4671,10 +4671,10 @@
       <c r="C44" s="118" t="inlineStr"/>
       <c r="D44" s="118" t="inlineStr"/>
       <c r="E44" s="66" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
+      <c r="F44" s="0" t="inlineStr"/>
       <c r="G44" s="118" t="inlineStr">
         <is>
-          <t>Not automated (proposed, gap-derived). Priority: Medium. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-46.</t>
+          <t>✅ Automated (Playwright): test_worker_gaps.py::test_src_w_46_worker_profile_kpis</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4692,7 @@
       <c r="C45" s="118" t="inlineStr"/>
       <c r="D45" s="118" t="inlineStr"/>
       <c r="E45" s="66" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
+      <c r="F45" s="0" t="inlineStr"/>
       <c r="G45" s="118" t="inlineStr">
         <is>
           <t>Not automated (proposed, gap-derived). Priority: High. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-47.</t>
@@ -4713,7 +4713,7 @@
       <c r="C46" s="118" t="inlineStr"/>
       <c r="D46" s="118" t="inlineStr"/>
       <c r="E46" s="66" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
+      <c r="F46" s="0" t="inlineStr"/>
       <c r="G46" s="118" t="inlineStr">
         <is>
           <t>Not automated (proposed, gap-derived). Priority: Medium. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-48.</t>
@@ -4734,10 +4734,10 @@
       <c r="C47" s="118" t="inlineStr"/>
       <c r="D47" s="118" t="inlineStr"/>
       <c r="E47" s="66" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
+      <c r="F47" s="0" t="inlineStr"/>
       <c r="G47" s="118" t="inlineStr">
         <is>
-          <t>Not automated (proposed, gap-derived). Priority: Medium. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-49.</t>
+          <t>✅ Automated (positive - tab present + reachable under MICROPLANNING): test_worker_gaps.py::test_src_w_49_work_area_tab_present. Off-state (absent + 404) needs a non-microplanning opp.</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       <c r="C48" s="118" t="inlineStr"/>
       <c r="D48" s="118" t="inlineStr"/>
       <c r="E48" s="66" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
+      <c r="F48" s="0" t="inlineStr"/>
       <c r="G48" s="118" t="inlineStr">
         <is>
           <t>Not automated (proposed, gap-derived). Priority: Medium. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-50.</t>
@@ -4776,7 +4776,7 @@
       <c r="C49" s="118" t="inlineStr"/>
       <c r="D49" s="118" t="inlineStr"/>
       <c r="E49" s="66" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
+      <c r="F49" s="0" t="inlineStr"/>
       <c r="G49" s="118" t="inlineStr">
         <is>
           <t>Not automated (proposed, gap-derived). Priority: Medium. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-51.</t>
@@ -4797,10 +4797,10 @@
       <c r="C50" s="118" t="inlineStr"/>
       <c r="D50" s="118" t="inlineStr"/>
       <c r="E50" s="66" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
+      <c r="F50" s="0" t="inlineStr"/>
       <c r="G50" s="118" t="inlineStr">
         <is>
-          <t>Not automated (proposed, gap-derived). Priority: Low. Action: Add to MTP only (eng-covered). Source: Gap Analysis GAP-SRC-W-52.</t>
+          <t>✅ Automated (partial - currency-suffixed headers): test_worker_gaps.py::test_src_w_52_payments_currency_headers. Footer sums / import cache-lock eng-covered.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automate gap cases GAP-SRC-W-47/48 + note _51 coverage (worker gaps, group 3)
- _47 (viewer half): a Connect-native viewer cannot add workers - the Add Worker
  control is disabled/absent on the workers page (direct viewer sign-in, like
  OD_21). has_ended half needs an ended opp.
- _48 (partial): the suspended-users list shows a 'Revoke suspension' column and
  lists the suspended worker (Map_08). Suspend-modal content + re-suspend
  idempotency deferred (needs a reliable path to the modal).
- _51: the count-breakdown popups are already covered by WLV_4/WLV_5 (per-worker
  and Total/footer); the Duplicate bucket + empty state need specific data.

Plan-sheet comments updated for _47/_48/_51. Validated headed: 2/2 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -4695,7 +4695,7 @@
       <c r="F45" s="0" t="inlineStr"/>
       <c r="G45" s="118" t="inlineStr">
         <is>
-          <t>Not automated (proposed, gap-derived). Priority: High. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-47.</t>
+          <t>✅ Automated (viewer half - Add Worker gated for a viewer): test_worker_gaps.py::test_src_w_47_viewer_read_only_gating. has_ended half needs an ended opp.</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       <c r="F46" s="0" t="inlineStr"/>
       <c r="G46" s="118" t="inlineStr">
         <is>
-          <t>Not automated (proposed, gap-derived). Priority: Medium. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-48.</t>
+          <t>✅ Automated (suspended-users list Revoke column + listing): test_worker_gaps.py::test_src_w_48_suspended_users_list. Suspend-modal content + re-suspend idempotency deferred (modal path).</t>
         </is>
       </c>
     </row>
@@ -4779,7 +4779,7 @@
       <c r="F49" s="0" t="inlineStr"/>
       <c r="G49" s="118" t="inlineStr">
         <is>
-          <t>Not automated (proposed, gap-derived). Priority: Medium. Action: Add to MTP + Automate (confirm w/ eng). Source: Gap Analysis GAP-SRC-W-51.</t>
+          <t>✅ Covered by WLV_4/WLV_5 count-breakdown popups (test_worker_list_view.py per-worker + Total/footer). Duplicate bucket + "No flagged visits" empty state need specific data - deferred.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automate Connect_worker_06/_09/_13 with Anshu's seeded data (Batch C)
Anshu added a resolved not-found worker (+74261291230, status "User not found")
and a real registered number for the cooldown (+919000696488) to
Worker_Lifecycle_Automation.

- _06: a not-found user shows "User not found" with no display name - only the
  mobile number (Name column "—"). Works for fresh or old invites.
- _13: the not-found user is deletable (Delete control enables on selection);
  not executed, to preserve the seeded worker (_08 already proves delete works).
- _09: resending the registered number within 24h is refused - "...skipped, as
  they were sent in the last 24 hours". Skip = no SMS. Relies on the invite
  staying <24h old (documented in the test/plan).

Logged in the MTP ledger; plan-tab comments updated. Validated headed: 3/3 pass.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_plans/CCC_Web_Platform_MTP.xlsx
+++ b/test_plans/CCC_Web_Platform_MTP.xlsx
@@ -3545,7 +3545,7 @@
       <c r="F9" s="104" t="n"/>
       <c r="G9" s="68" t="inlineStr">
         <is>
-          <t>⏳ Not automated - not-found "mobile under Name" resolves asynchronously (SMS delivery callback); a freshly-invited number shows "—". Needs a resolved not-found worker seeded (requested from data setup).</t>
+          <t>✅ Automated (Playwright): test_worker_lifecycle.py::test_connect_worker_06_not_found_display (seeded not-found +74261291230, status "User not found", "—" under Name).</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3645,7 @@
       <c r="F12" s="85" t="n"/>
       <c r="G12" s="88" t="inlineStr">
         <is>
-          <t>🔴 Manual only - demo/reserved numbers do NOT enforce the 24h resend cooldown (per data setup); needs a real number to verify.</t>
+          <t>✅ Automated (Playwright): test_worker_lifecycle.py::test_connect_worker_09_resend_cooldown (real number +919000696488 -&gt; "sent in the last 24 hours"). NOTE: relies on the invite staying &lt;24h old; refresh if it flips.</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3778,7 @@
       <c r="F16" s="85" t="n"/>
       <c r="G16" s="88" t="inlineStr">
         <is>
-          <t>⏳ Not automated - delete not-found shares the async not-found dependency as _06; needs a resolved not-found worker seeded.</t>
+          <t>✅ Automated (Playwright): test_worker_lifecycle.py::test_connect_worker_13_not_found_deletable (Delete affordance on the seeded not-found user; not executed to preserve the seed).</t>
         </is>
       </c>
     </row>
@@ -20447,7 +20447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G336"/>
+  <dimension ref="A1:G339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="148" min="1" max="1"/>
@@ -32886,6 +32886,117 @@
         </is>
       </c>
       <c r="G336" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_06</t>
+        </is>
+      </c>
+      <c r="B337" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C337" s="171" t="inlineStr">
+        <is>
+          <t>Verify a not-found (unregistered) user shows "User not found" with no name - only the mobile number</t>
+        </is>
+      </c>
+      <c r="D337" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E337" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_06_not_found_display</t>
+        </is>
+      </c>
+      <c r="F337" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C - Anshu data 2 (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G337" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_09</t>
+        </is>
+      </c>
+      <c r="B338" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C338" s="171" t="inlineStr">
+        <is>
+          <t>Verify user is not able to resend the invite within 24h (cooldown) - real number</t>
+        </is>
+      </c>
+      <c r="D338" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E338" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_09_resend_cooldown</t>
+        </is>
+      </c>
+      <c r="F338" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C - Anshu data 2 (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G338" s="171" t="inlineStr">
+        <is>
+          <t>Already automated (n/a)</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="171" t="inlineStr">
+        <is>
+          <t>Connect_worker_13</t>
+        </is>
+      </c>
+      <c r="B339" s="171" t="inlineStr">
+        <is>
+          <t>Connect workers page</t>
+        </is>
+      </c>
+      <c r="C339" s="171" t="inlineStr">
+        <is>
+          <t>Verify user is able to delete not-found users (Delete affordance; not executed to preserve seed)</t>
+        </is>
+      </c>
+      <c r="D339" s="171" t="inlineStr">
+        <is>
+          <t>🟢 Already automated</t>
+        </is>
+      </c>
+      <c r="E339" s="171" t="inlineStr">
+        <is>
+          <t>test_worker_lifecycle.py::test_connect_worker_13_not_found_deletable</t>
+        </is>
+      </c>
+      <c r="F339" s="171" t="inlineStr">
+        <is>
+          <t>Connect Workers Batch C - Anshu data 2 (Worker_Lifecycle_Automation, 2026-09-10)</t>
+        </is>
+      </c>
+      <c r="G339" s="171" t="inlineStr">
         <is>
           <t>Already automated (n/a)</t>
         </is>

</xml_diff>